<commit_message>
ASN ref, FOB and Fs modified on vbkreq
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="131">
   <si>
     <t>PO_Number</t>
   </si>
@@ -108,13 +108,13 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>500034207447</t>
-  </si>
-  <si>
-    <t>49870000001015</t>
-  </si>
-  <si>
-    <t>148609059</t>
+    <t>500034231405</t>
+  </si>
+  <si>
+    <t>45870000003656</t>
+  </si>
+  <si>
+    <t>123478460</t>
   </si>
   <si>
     <t>CFS</t>
@@ -135,6 +135,27 @@
     <t>N/A</t>
   </si>
   <si>
+    <t>123478461</t>
+  </si>
+  <si>
+    <t>123478462</t>
+  </si>
+  <si>
+    <t>123478463</t>
+  </si>
+  <si>
+    <t>123478464</t>
+  </si>
+  <si>
+    <t>123478465</t>
+  </si>
+  <si>
+    <t>123478466</t>
+  </si>
+  <si>
+    <t>123478467</t>
+  </si>
+  <si>
     <t>orderId</t>
   </si>
   <si>
@@ -171,16 +192,16 @@
     <t>incoterms</t>
   </si>
   <si>
-    <t>Difuzed - FOB</t>
-  </si>
-  <si>
-    <t>2002900003</t>
-  </si>
-  <si>
-    <t>Ozon Tekstil Konfeksiyon San Ve Tic AS Sivas</t>
-  </si>
-  <si>
-    <t>F103330</t>
+    <t>Tudorknight Limited (OB)</t>
+  </si>
+  <si>
+    <t>1100004812</t>
+  </si>
+  <si>
+    <t>Dummy Factory</t>
+  </si>
+  <si>
+    <t>9999</t>
   </si>
   <si>
     <t>FC01 Barnsley</t>
@@ -192,7 +213,7 @@
     <t>3</t>
   </si>
   <si>
-    <t>GERBE</t>
+    <t>TURIS</t>
   </si>
   <si>
     <t>FOB</t>
@@ -213,9 +234,6 @@
     <t>shipmentRef</t>
   </si>
   <si>
-    <t>148609060</t>
-  </si>
-  <si>
     <t>Booking_Ref</t>
   </si>
   <si>
@@ -303,10 +321,10 @@
     <t>European Nom Carrier</t>
   </si>
   <si>
-    <t>148609056</t>
-  </si>
-  <si>
-    <t>T&amp;R POKEMON ESPEON</t>
+    <t>123478454</t>
+  </si>
+  <si>
+    <t>HONEY REV</t>
   </si>
   <si>
     <t>30</t>
@@ -786,7 +804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="30" width="22" customWidth="1"/>
@@ -937,13 +955,13 @@
         <v>1.4</v>
       </c>
       <c r="R2">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="S2">
         <v>0.072</v>
       </c>
       <c r="T2">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="U2" t="s">
         <v>36</v>
@@ -973,6 +991,650 @@
         <v>0</v>
       </c>
       <c r="AD2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46192</v>
+      </c>
+      <c r="G3" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M3">
+        <v>60</v>
+      </c>
+      <c r="N3">
+        <v>30</v>
+      </c>
+      <c r="O3">
+        <v>40</v>
+      </c>
+      <c r="P3">
+        <v>1.4</v>
+      </c>
+      <c r="Q3">
+        <v>2.8</v>
+      </c>
+      <c r="R3">
+        <v>750</v>
+      </c>
+      <c r="S3">
+        <v>0.144</v>
+      </c>
+      <c r="T3">
+        <v>125</v>
+      </c>
+      <c r="U3" t="s">
+        <v>36</v>
+      </c>
+      <c r="V3" t="s">
+        <v>37</v>
+      </c>
+      <c r="W3" t="s">
+        <v>34</v>
+      </c>
+      <c r="X3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46192</v>
+      </c>
+      <c r="G4" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M4">
+        <v>60</v>
+      </c>
+      <c r="N4">
+        <v>30</v>
+      </c>
+      <c r="O4">
+        <v>40</v>
+      </c>
+      <c r="P4">
+        <v>1.4</v>
+      </c>
+      <c r="Q4">
+        <v>4.199999999999999</v>
+      </c>
+      <c r="R4">
+        <v>1375</v>
+      </c>
+      <c r="S4">
+        <v>0.21599999999999997</v>
+      </c>
+      <c r="T4">
+        <v>125</v>
+      </c>
+      <c r="U4" t="s">
+        <v>36</v>
+      </c>
+      <c r="V4" t="s">
+        <v>37</v>
+      </c>
+      <c r="W4" t="s">
+        <v>34</v>
+      </c>
+      <c r="X4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>16</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46192</v>
+      </c>
+      <c r="G5" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5">
+        <v>60</v>
+      </c>
+      <c r="N5">
+        <v>30</v>
+      </c>
+      <c r="O5">
+        <v>40</v>
+      </c>
+      <c r="P5">
+        <v>1.4</v>
+      </c>
+      <c r="Q5">
+        <v>5.6</v>
+      </c>
+      <c r="R5">
+        <v>2000</v>
+      </c>
+      <c r="S5">
+        <v>0.288</v>
+      </c>
+      <c r="T5">
+        <v>125</v>
+      </c>
+      <c r="U5" t="s">
+        <v>36</v>
+      </c>
+      <c r="V5" t="s">
+        <v>37</v>
+      </c>
+      <c r="W5" t="s">
+        <v>34</v>
+      </c>
+      <c r="X5" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>21</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46192</v>
+      </c>
+      <c r="G6" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" t="s">
+        <v>35</v>
+      </c>
+      <c r="M6">
+        <v>60</v>
+      </c>
+      <c r="N6">
+        <v>30</v>
+      </c>
+      <c r="O6">
+        <v>40</v>
+      </c>
+      <c r="P6">
+        <v>1.4</v>
+      </c>
+      <c r="Q6">
+        <v>7</v>
+      </c>
+      <c r="R6">
+        <v>2625</v>
+      </c>
+      <c r="S6">
+        <v>0.36</v>
+      </c>
+      <c r="T6">
+        <v>125</v>
+      </c>
+      <c r="U6" t="s">
+        <v>36</v>
+      </c>
+      <c r="V6" t="s">
+        <v>37</v>
+      </c>
+      <c r="W6" t="s">
+        <v>34</v>
+      </c>
+      <c r="X6" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>26</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46192</v>
+      </c>
+      <c r="G7" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" t="s">
+        <v>35</v>
+      </c>
+      <c r="M7">
+        <v>60</v>
+      </c>
+      <c r="N7">
+        <v>30</v>
+      </c>
+      <c r="O7">
+        <v>40</v>
+      </c>
+      <c r="P7">
+        <v>1.4</v>
+      </c>
+      <c r="Q7">
+        <v>8.399999999999999</v>
+      </c>
+      <c r="R7">
+        <v>3250</v>
+      </c>
+      <c r="S7">
+        <v>0.43199999999999994</v>
+      </c>
+      <c r="T7">
+        <v>125</v>
+      </c>
+      <c r="U7" t="s">
+        <v>36</v>
+      </c>
+      <c r="V7" t="s">
+        <v>37</v>
+      </c>
+      <c r="W7" t="s">
+        <v>34</v>
+      </c>
+      <c r="X7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB7">
+        <v>0</v>
+      </c>
+      <c r="AC7">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8">
+        <v>31</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46192</v>
+      </c>
+      <c r="G8" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H8" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K8" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8">
+        <v>60</v>
+      </c>
+      <c r="N8">
+        <v>30</v>
+      </c>
+      <c r="O8">
+        <v>40</v>
+      </c>
+      <c r="P8">
+        <v>1.4</v>
+      </c>
+      <c r="Q8">
+        <v>9.799999999999999</v>
+      </c>
+      <c r="R8">
+        <v>3875</v>
+      </c>
+      <c r="S8">
+        <v>0.504</v>
+      </c>
+      <c r="T8">
+        <v>125</v>
+      </c>
+      <c r="U8" t="s">
+        <v>36</v>
+      </c>
+      <c r="V8" t="s">
+        <v>37</v>
+      </c>
+      <c r="W8" t="s">
+        <v>34</v>
+      </c>
+      <c r="X8" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB8">
+        <v>0</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>36</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46192</v>
+      </c>
+      <c r="G9" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H9" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" t="s">
+        <v>35</v>
+      </c>
+      <c r="M9">
+        <v>60</v>
+      </c>
+      <c r="N9">
+        <v>30</v>
+      </c>
+      <c r="O9">
+        <v>40</v>
+      </c>
+      <c r="P9">
+        <v>1.4</v>
+      </c>
+      <c r="Q9">
+        <v>11.2</v>
+      </c>
+      <c r="R9" t="s">
+        <v>34</v>
+      </c>
+      <c r="S9">
+        <v>0.576</v>
+      </c>
+      <c r="T9" t="s">
+        <v>34</v>
+      </c>
+      <c r="U9" t="s">
+        <v>36</v>
+      </c>
+      <c r="V9" t="s">
+        <v>37</v>
+      </c>
+      <c r="W9" t="s">
+        <v>34</v>
+      </c>
+      <c r="X9" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB9">
+        <v>0</v>
+      </c>
+      <c r="AC9">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="s">
         <v>34</v>
       </c>
     </row>
@@ -992,40 +1654,40 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1033,16 +1695,16 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F2" t="s">
         <v>34</v>
@@ -1051,19 +1713,19 @@
         <v>34</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="J2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="K2" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="L2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1074,7 +1736,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="22" customWidth="1"/>
@@ -1082,25 +1744,25 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1108,7 +1770,7 @@
         <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
         <v>34</v>
@@ -1117,7 +1779,7 @@
         <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1131,7 +1793,7 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
         <v>34</v>
@@ -1140,12 +1802,150 @@
         <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1157,7 +1957,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BE2"/>
+  <dimension ref="A1:BE9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="57" width="22" customWidth="1"/>
@@ -1165,7 +1965,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1174,79 +1974,79 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="AC1" s="1" t="s">
         <v>8</v>
@@ -1330,10 +2130,10 @@
         <v>22</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:57" x14ac:dyDescent="0.25">
@@ -1347,16 +2147,16 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="H2" t="s">
         <v>34</v>
@@ -1377,10 +2177,10 @@
         <v>34</v>
       </c>
       <c r="N2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="O2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="P2" t="s">
         <v>34</v>
@@ -1401,25 +2201,25 @@
         <v>34</v>
       </c>
       <c r="V2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="W2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="X2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="Y2" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="Z2" t="s">
         <v>32</v>
       </c>
       <c r="AA2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="AB2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="AC2" t="s">
         <v>34</v>
@@ -1452,13 +2252,13 @@
         <v>1</v>
       </c>
       <c r="AM2">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="AN2" s="3">
         <v>1.4</v>
       </c>
       <c r="AO2" s="3">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="AP2" s="3">
         <v>0.072</v>
@@ -1503,10 +2303,1221 @@
         <v>34</v>
       </c>
       <c r="BD2" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" t="s">
         <v>59</v>
       </c>
-      <c r="BE2" t="s">
-        <v>97</v>
+      <c r="F3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" t="s">
+        <v>62</v>
+      </c>
+      <c r="O3" t="s">
+        <v>63</v>
+      </c>
+      <c r="P3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" t="s">
+        <v>34</v>
+      </c>
+      <c r="S3" t="s">
+        <v>34</v>
+      </c>
+      <c r="T3" t="s">
+        <v>34</v>
+      </c>
+      <c r="U3" t="s">
+        <v>34</v>
+      </c>
+      <c r="V3" t="s">
+        <v>99</v>
+      </c>
+      <c r="W3" t="s">
+        <v>64</v>
+      </c>
+      <c r="X3" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG3" s="3">
+        <v>60</v>
+      </c>
+      <c r="AH3" s="3">
+        <v>30</v>
+      </c>
+      <c r="AI3" s="3">
+        <v>40</v>
+      </c>
+      <c r="AJ3" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="AK3">
+        <v>2</v>
+      </c>
+      <c r="AL3">
+        <v>6</v>
+      </c>
+      <c r="AM3">
+        <v>125</v>
+      </c>
+      <c r="AN3" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="AO3" s="3">
+        <v>750</v>
+      </c>
+      <c r="AP3" s="3">
+        <v>0.144</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AU3" s="2">
+        <v>46192</v>
+      </c>
+      <c r="AV3" s="2">
+        <v>46193</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AY3">
+        <v>0</v>
+      </c>
+      <c r="AZ3">
+        <v>0</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>34</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>34</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" t="s">
+        <v>34</v>
+      </c>
+      <c r="M4" t="s">
+        <v>34</v>
+      </c>
+      <c r="N4" t="s">
+        <v>62</v>
+      </c>
+      <c r="O4" t="s">
+        <v>63</v>
+      </c>
+      <c r="P4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>34</v>
+      </c>
+      <c r="R4" t="s">
+        <v>34</v>
+      </c>
+      <c r="S4" t="s">
+        <v>34</v>
+      </c>
+      <c r="T4" t="s">
+        <v>34</v>
+      </c>
+      <c r="U4" t="s">
+        <v>34</v>
+      </c>
+      <c r="V4" t="s">
+        <v>99</v>
+      </c>
+      <c r="W4" t="s">
+        <v>64</v>
+      </c>
+      <c r="X4" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG4" s="3">
+        <v>60</v>
+      </c>
+      <c r="AH4" s="3">
+        <v>30</v>
+      </c>
+      <c r="AI4" s="3">
+        <v>40</v>
+      </c>
+      <c r="AJ4" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="AK4">
+        <v>3</v>
+      </c>
+      <c r="AL4">
+        <v>11</v>
+      </c>
+      <c r="AM4">
+        <v>125</v>
+      </c>
+      <c r="AN4" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="AO4" s="3">
+        <v>1375</v>
+      </c>
+      <c r="AP4" s="3">
+        <v>0.216</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT4" t="s">
+        <v>33</v>
+      </c>
+      <c r="AU4" s="2">
+        <v>46192</v>
+      </c>
+      <c r="AV4" s="2">
+        <v>46193</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AY4">
+        <v>0</v>
+      </c>
+      <c r="AZ4">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>34</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>34</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N5" t="s">
+        <v>62</v>
+      </c>
+      <c r="O5" t="s">
+        <v>63</v>
+      </c>
+      <c r="P5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>34</v>
+      </c>
+      <c r="R5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T5" t="s">
+        <v>34</v>
+      </c>
+      <c r="U5" t="s">
+        <v>34</v>
+      </c>
+      <c r="V5" t="s">
+        <v>99</v>
+      </c>
+      <c r="W5" t="s">
+        <v>64</v>
+      </c>
+      <c r="X5" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG5" s="3">
+        <v>60</v>
+      </c>
+      <c r="AH5" s="3">
+        <v>30</v>
+      </c>
+      <c r="AI5" s="3">
+        <v>40</v>
+      </c>
+      <c r="AJ5" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="AK5">
+        <v>4</v>
+      </c>
+      <c r="AL5">
+        <v>16</v>
+      </c>
+      <c r="AM5">
+        <v>125</v>
+      </c>
+      <c r="AN5" s="3">
+        <v>5.6</v>
+      </c>
+      <c r="AO5" s="3">
+        <v>2000</v>
+      </c>
+      <c r="AP5" s="3">
+        <v>0.288</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AU5" s="2">
+        <v>46192</v>
+      </c>
+      <c r="AV5" s="2">
+        <v>46193</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AY5">
+        <v>0</v>
+      </c>
+      <c r="AZ5">
+        <v>0</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>34</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>34</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" t="s">
+        <v>62</v>
+      </c>
+      <c r="O6" t="s">
+        <v>63</v>
+      </c>
+      <c r="P6" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" t="s">
+        <v>34</v>
+      </c>
+      <c r="T6" t="s">
+        <v>34</v>
+      </c>
+      <c r="U6" t="s">
+        <v>34</v>
+      </c>
+      <c r="V6" t="s">
+        <v>99</v>
+      </c>
+      <c r="W6" t="s">
+        <v>64</v>
+      </c>
+      <c r="X6" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG6" s="3">
+        <v>60</v>
+      </c>
+      <c r="AH6" s="3">
+        <v>30</v>
+      </c>
+      <c r="AI6" s="3">
+        <v>40</v>
+      </c>
+      <c r="AJ6" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="AK6">
+        <v>5</v>
+      </c>
+      <c r="AL6">
+        <v>21</v>
+      </c>
+      <c r="AM6">
+        <v>125</v>
+      </c>
+      <c r="AN6" s="3">
+        <v>7</v>
+      </c>
+      <c r="AO6" s="3">
+        <v>2625</v>
+      </c>
+      <c r="AP6" s="3">
+        <v>0.36</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT6" t="s">
+        <v>33</v>
+      </c>
+      <c r="AU6" s="2">
+        <v>46192</v>
+      </c>
+      <c r="AV6" s="2">
+        <v>46193</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AX6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AY6">
+        <v>0</v>
+      </c>
+      <c r="AZ6">
+        <v>0</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>34</v>
+      </c>
+      <c r="BB6" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC6" t="s">
+        <v>34</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" t="s">
+        <v>34</v>
+      </c>
+      <c r="M7" t="s">
+        <v>34</v>
+      </c>
+      <c r="N7" t="s">
+        <v>62</v>
+      </c>
+      <c r="O7" t="s">
+        <v>63</v>
+      </c>
+      <c r="P7" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>34</v>
+      </c>
+      <c r="R7" t="s">
+        <v>34</v>
+      </c>
+      <c r="S7" t="s">
+        <v>34</v>
+      </c>
+      <c r="T7" t="s">
+        <v>34</v>
+      </c>
+      <c r="U7" t="s">
+        <v>34</v>
+      </c>
+      <c r="V7" t="s">
+        <v>99</v>
+      </c>
+      <c r="W7" t="s">
+        <v>64</v>
+      </c>
+      <c r="X7" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG7" s="3">
+        <v>60</v>
+      </c>
+      <c r="AH7" s="3">
+        <v>30</v>
+      </c>
+      <c r="AI7" s="3">
+        <v>40</v>
+      </c>
+      <c r="AJ7" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="AK7">
+        <v>6</v>
+      </c>
+      <c r="AL7">
+        <v>26</v>
+      </c>
+      <c r="AM7">
+        <v>125</v>
+      </c>
+      <c r="AN7" s="3">
+        <v>8.4</v>
+      </c>
+      <c r="AO7" s="3">
+        <v>3250</v>
+      </c>
+      <c r="AP7" s="3">
+        <v>0.432</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AU7" s="2">
+        <v>46192</v>
+      </c>
+      <c r="AV7" s="2">
+        <v>46193</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AY7">
+        <v>0</v>
+      </c>
+      <c r="AZ7">
+        <v>0</v>
+      </c>
+      <c r="BA7" t="s">
+        <v>34</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC7" t="s">
+        <v>34</v>
+      </c>
+      <c r="BD7" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K8" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N8" t="s">
+        <v>62</v>
+      </c>
+      <c r="O8" t="s">
+        <v>63</v>
+      </c>
+      <c r="P8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>34</v>
+      </c>
+      <c r="R8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S8" t="s">
+        <v>34</v>
+      </c>
+      <c r="T8" t="s">
+        <v>34</v>
+      </c>
+      <c r="U8" t="s">
+        <v>34</v>
+      </c>
+      <c r="V8" t="s">
+        <v>99</v>
+      </c>
+      <c r="W8" t="s">
+        <v>64</v>
+      </c>
+      <c r="X8" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG8" s="3">
+        <v>60</v>
+      </c>
+      <c r="AH8" s="3">
+        <v>30</v>
+      </c>
+      <c r="AI8" s="3">
+        <v>40</v>
+      </c>
+      <c r="AJ8" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="AK8">
+        <v>7</v>
+      </c>
+      <c r="AL8">
+        <v>31</v>
+      </c>
+      <c r="AM8">
+        <v>125</v>
+      </c>
+      <c r="AN8" s="3">
+        <v>9.8</v>
+      </c>
+      <c r="AO8" s="3">
+        <v>3875</v>
+      </c>
+      <c r="AP8" s="3">
+        <v>0.504</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT8" t="s">
+        <v>33</v>
+      </c>
+      <c r="AU8" s="2">
+        <v>46192</v>
+      </c>
+      <c r="AV8" s="2">
+        <v>46193</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AX8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AY8">
+        <v>0</v>
+      </c>
+      <c r="AZ8">
+        <v>0</v>
+      </c>
+      <c r="BA8" t="s">
+        <v>34</v>
+      </c>
+      <c r="BB8" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC8" t="s">
+        <v>34</v>
+      </c>
+      <c r="BD8" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M9" t="s">
+        <v>34</v>
+      </c>
+      <c r="N9" t="s">
+        <v>62</v>
+      </c>
+      <c r="O9" t="s">
+        <v>63</v>
+      </c>
+      <c r="P9" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>34</v>
+      </c>
+      <c r="R9" t="s">
+        <v>34</v>
+      </c>
+      <c r="S9" t="s">
+        <v>34</v>
+      </c>
+      <c r="T9" t="s">
+        <v>34</v>
+      </c>
+      <c r="U9" t="s">
+        <v>34</v>
+      </c>
+      <c r="V9" t="s">
+        <v>99</v>
+      </c>
+      <c r="W9" t="s">
+        <v>64</v>
+      </c>
+      <c r="X9" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG9" s="3">
+        <v>60</v>
+      </c>
+      <c r="AH9" s="3">
+        <v>30</v>
+      </c>
+      <c r="AI9" s="3">
+        <v>40</v>
+      </c>
+      <c r="AJ9" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="AK9">
+        <v>8</v>
+      </c>
+      <c r="AL9">
+        <v>36</v>
+      </c>
+      <c r="AM9">
+        <v>0</v>
+      </c>
+      <c r="AN9" s="3">
+        <v>11.2</v>
+      </c>
+      <c r="AO9" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="3">
+        <v>0.576</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>36</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT9" t="s">
+        <v>33</v>
+      </c>
+      <c r="AU9" s="2">
+        <v>46192</v>
+      </c>
+      <c r="AV9" s="2">
+        <v>46193</v>
+      </c>
+      <c r="AW9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AX9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AY9">
+        <v>0</v>
+      </c>
+      <c r="AZ9">
+        <v>0</v>
+      </c>
+      <c r="BA9" t="s">
+        <v>34</v>
+      </c>
+      <c r="BB9" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC9" t="s">
+        <v>34</v>
+      </c>
+      <c r="BD9" t="s">
+        <v>66</v>
+      </c>
+      <c r="BE9" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1528,16 +3539,16 @@
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1559,7 +3570,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1576,7 +3587,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1593,7 +3604,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1610,7 +3621,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1627,7 +3638,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1644,7 +3655,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1661,7 +3672,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1678,7 +3689,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1695,7 +3706,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1712,7 +3723,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1729,7 +3740,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1746,7 +3757,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1763,7 +3774,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1780,7 +3791,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1797,7 +3808,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1814,7 +3825,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -1831,12 +3842,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1855,22 +3866,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bible ignored from git
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="132">
   <si>
     <t>PO_Number</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Loading_Port_LOCODE</t>
+  </si>
+  <si>
+    <t>F1_ID</t>
   </si>
   <si>
     <t>Product_Style</t>
@@ -1957,13 +1960,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BE9"/>
+  <dimension ref="A1:BF9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="57" width="22" customWidth="1"/>
+    <col min="1" max="58" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:57" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>72</v>
       </c>
@@ -2040,103 +2043,106 @@
         <v>94</v>
       </c>
       <c r="Z1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>96</v>
       </c>
       <c r="AC1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AD1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="BE1" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="2" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF1" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -2201,28 +2207,28 @@
         <v>34</v>
       </c>
       <c r="V2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W2" t="s">
         <v>64</v>
       </c>
       <c r="X2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y2" t="s">
         <v>65</v>
       </c>
       <c r="Z2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA2" t="s">
         <v>32</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>101</v>
       </c>
       <c r="AB2" t="s">
         <v>102</v>
       </c>
       <c r="AC2" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD2" t="s">
         <v>34</v>
@@ -2231,70 +2237,70 @@
         <v>34</v>
       </c>
       <c r="AF2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG2" t="s">
         <v>35</v>
       </c>
-      <c r="AG2" s="3">
+      <c r="AH2" s="3">
         <v>60</v>
       </c>
-      <c r="AH2" s="3">
-        <v>30</v>
-      </c>
       <c r="AI2" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ2" s="3">
         <v>40</v>
       </c>
-      <c r="AJ2" s="3">
+      <c r="AK2" s="3">
         <v>1.4</v>
-      </c>
-      <c r="AK2">
-        <v>1</v>
       </c>
       <c r="AL2">
         <v>1</v>
       </c>
       <c r="AM2">
+        <v>1</v>
+      </c>
+      <c r="AN2">
         <v>125</v>
       </c>
-      <c r="AN2" s="3">
+      <c r="AO2" s="3">
         <v>1.4</v>
       </c>
-      <c r="AO2" s="3">
+      <c r="AP2" s="3">
         <v>125</v>
       </c>
-      <c r="AP2" s="3">
+      <c r="AQ2" s="3">
         <v>0.072</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AR2" t="s">
         <v>36</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AS2" t="s">
         <v>37</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AT2" t="s">
         <v>38</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AU2" t="s">
         <v>33</v>
       </c>
-      <c r="AU2" s="2">
+      <c r="AV2" s="2">
         <v>46192</v>
       </c>
-      <c r="AV2" s="2">
+      <c r="AW2" s="2">
         <v>46193</v>
       </c>
-      <c r="AW2" t="s">
-        <v>34</v>
-      </c>
       <c r="AX2" t="s">
         <v>34</v>
       </c>
-      <c r="AY2">
-        <v>0</v>
+      <c r="AY2" t="s">
+        <v>34</v>
       </c>
       <c r="AZ2">
         <v>0</v>
       </c>
-      <c r="BA2" t="s">
-        <v>34</v>
+      <c r="BA2">
+        <v>0</v>
       </c>
       <c r="BB2" t="s">
         <v>34</v>
@@ -2303,13 +2309,16 @@
         <v>34</v>
       </c>
       <c r="BD2" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE2" t="s">
         <v>66</v>
       </c>
-      <c r="BE2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="3" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -2374,28 +2383,28 @@
         <v>34</v>
       </c>
       <c r="V3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W3" t="s">
         <v>64</v>
       </c>
       <c r="X3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y3" t="s">
         <v>65</v>
       </c>
       <c r="Z3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA3" t="s">
         <v>39</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>101</v>
       </c>
       <c r="AB3" t="s">
         <v>102</v>
       </c>
       <c r="AC3" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD3" t="s">
         <v>34</v>
@@ -2404,70 +2413,70 @@
         <v>34</v>
       </c>
       <c r="AF3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG3" t="s">
         <v>35</v>
       </c>
-      <c r="AG3" s="3">
+      <c r="AH3" s="3">
         <v>60</v>
       </c>
-      <c r="AH3" s="3">
-        <v>30</v>
-      </c>
       <c r="AI3" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ3" s="3">
         <v>40</v>
       </c>
-      <c r="AJ3" s="3">
+      <c r="AK3" s="3">
         <v>1.4</v>
       </c>
-      <c r="AK3">
+      <c r="AL3">
         <v>2</v>
       </c>
-      <c r="AL3">
+      <c r="AM3">
         <v>6</v>
       </c>
-      <c r="AM3">
+      <c r="AN3">
         <v>125</v>
       </c>
-      <c r="AN3" s="3">
+      <c r="AO3" s="3">
         <v>2.8</v>
       </c>
-      <c r="AO3" s="3">
+      <c r="AP3" s="3">
         <v>750</v>
       </c>
-      <c r="AP3" s="3">
+      <c r="AQ3" s="3">
         <v>0.144</v>
       </c>
-      <c r="AQ3" t="s">
+      <c r="AR3" t="s">
         <v>36</v>
       </c>
-      <c r="AR3" t="s">
+      <c r="AS3" t="s">
         <v>37</v>
       </c>
-      <c r="AS3" t="s">
+      <c r="AT3" t="s">
         <v>38</v>
       </c>
-      <c r="AT3" t="s">
+      <c r="AU3" t="s">
         <v>33</v>
       </c>
-      <c r="AU3" s="2">
+      <c r="AV3" s="2">
         <v>46192</v>
       </c>
-      <c r="AV3" s="2">
+      <c r="AW3" s="2">
         <v>46193</v>
       </c>
-      <c r="AW3" t="s">
-        <v>34</v>
-      </c>
       <c r="AX3" t="s">
         <v>34</v>
       </c>
-      <c r="AY3">
-        <v>0</v>
+      <c r="AY3" t="s">
+        <v>34</v>
       </c>
       <c r="AZ3">
         <v>0</v>
       </c>
-      <c r="BA3" t="s">
-        <v>34</v>
+      <c r="BA3">
+        <v>0</v>
       </c>
       <c r="BB3" t="s">
         <v>34</v>
@@ -2476,13 +2485,16 @@
         <v>34</v>
       </c>
       <c r="BD3" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE3" t="s">
         <v>66</v>
       </c>
-      <c r="BE3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -2547,28 +2559,28 @@
         <v>34</v>
       </c>
       <c r="V4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W4" t="s">
         <v>64</v>
       </c>
       <c r="X4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y4" t="s">
         <v>65</v>
       </c>
       <c r="Z4" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA4" t="s">
         <v>40</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>101</v>
       </c>
       <c r="AB4" t="s">
         <v>102</v>
       </c>
       <c r="AC4" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD4" t="s">
         <v>34</v>
@@ -2577,70 +2589,70 @@
         <v>34</v>
       </c>
       <c r="AF4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG4" t="s">
         <v>35</v>
       </c>
-      <c r="AG4" s="3">
+      <c r="AH4" s="3">
         <v>60</v>
       </c>
-      <c r="AH4" s="3">
-        <v>30</v>
-      </c>
       <c r="AI4" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ4" s="3">
         <v>40</v>
       </c>
-      <c r="AJ4" s="3">
+      <c r="AK4" s="3">
         <v>1.4</v>
       </c>
-      <c r="AK4">
+      <c r="AL4">
         <v>3</v>
       </c>
-      <c r="AL4">
+      <c r="AM4">
         <v>11</v>
       </c>
-      <c r="AM4">
+      <c r="AN4">
         <v>125</v>
       </c>
-      <c r="AN4" s="3">
+      <c r="AO4" s="3">
         <v>4.2</v>
       </c>
-      <c r="AO4" s="3">
+      <c r="AP4" s="3">
         <v>1375</v>
       </c>
-      <c r="AP4" s="3">
+      <c r="AQ4" s="3">
         <v>0.216</v>
       </c>
-      <c r="AQ4" t="s">
+      <c r="AR4" t="s">
         <v>36</v>
       </c>
-      <c r="AR4" t="s">
+      <c r="AS4" t="s">
         <v>37</v>
       </c>
-      <c r="AS4" t="s">
+      <c r="AT4" t="s">
         <v>38</v>
       </c>
-      <c r="AT4" t="s">
+      <c r="AU4" t="s">
         <v>33</v>
       </c>
-      <c r="AU4" s="2">
+      <c r="AV4" s="2">
         <v>46192</v>
       </c>
-      <c r="AV4" s="2">
+      <c r="AW4" s="2">
         <v>46193</v>
       </c>
-      <c r="AW4" t="s">
-        <v>34</v>
-      </c>
       <c r="AX4" t="s">
         <v>34</v>
       </c>
-      <c r="AY4">
-        <v>0</v>
+      <c r="AY4" t="s">
+        <v>34</v>
       </c>
       <c r="AZ4">
         <v>0</v>
       </c>
-      <c r="BA4" t="s">
-        <v>34</v>
+      <c r="BA4">
+        <v>0</v>
       </c>
       <c r="BB4" t="s">
         <v>34</v>
@@ -2649,13 +2661,16 @@
         <v>34</v>
       </c>
       <c r="BD4" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE4" t="s">
         <v>66</v>
       </c>
-      <c r="BE4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -2720,28 +2735,28 @@
         <v>34</v>
       </c>
       <c r="V5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W5" t="s">
         <v>64</v>
       </c>
       <c r="X5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y5" t="s">
         <v>65</v>
       </c>
       <c r="Z5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA5" t="s">
         <v>41</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>101</v>
       </c>
       <c r="AB5" t="s">
         <v>102</v>
       </c>
       <c r="AC5" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD5" t="s">
         <v>34</v>
@@ -2750,70 +2765,70 @@
         <v>34</v>
       </c>
       <c r="AF5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG5" t="s">
         <v>35</v>
       </c>
-      <c r="AG5" s="3">
+      <c r="AH5" s="3">
         <v>60</v>
       </c>
-      <c r="AH5" s="3">
-        <v>30</v>
-      </c>
       <c r="AI5" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ5" s="3">
         <v>40</v>
       </c>
-      <c r="AJ5" s="3">
+      <c r="AK5" s="3">
         <v>1.4</v>
       </c>
-      <c r="AK5">
+      <c r="AL5">
         <v>4</v>
       </c>
-      <c r="AL5">
+      <c r="AM5">
         <v>16</v>
       </c>
-      <c r="AM5">
+      <c r="AN5">
         <v>125</v>
       </c>
-      <c r="AN5" s="3">
+      <c r="AO5" s="3">
         <v>5.6</v>
       </c>
-      <c r="AO5" s="3">
+      <c r="AP5" s="3">
         <v>2000</v>
       </c>
-      <c r="AP5" s="3">
+      <c r="AQ5" s="3">
         <v>0.288</v>
       </c>
-      <c r="AQ5" t="s">
+      <c r="AR5" t="s">
         <v>36</v>
       </c>
-      <c r="AR5" t="s">
+      <c r="AS5" t="s">
         <v>37</v>
       </c>
-      <c r="AS5" t="s">
+      <c r="AT5" t="s">
         <v>38</v>
       </c>
-      <c r="AT5" t="s">
+      <c r="AU5" t="s">
         <v>33</v>
       </c>
-      <c r="AU5" s="2">
+      <c r="AV5" s="2">
         <v>46192</v>
       </c>
-      <c r="AV5" s="2">
+      <c r="AW5" s="2">
         <v>46193</v>
       </c>
-      <c r="AW5" t="s">
-        <v>34</v>
-      </c>
       <c r="AX5" t="s">
         <v>34</v>
       </c>
-      <c r="AY5">
-        <v>0</v>
+      <c r="AY5" t="s">
+        <v>34</v>
       </c>
       <c r="AZ5">
         <v>0</v>
       </c>
-      <c r="BA5" t="s">
-        <v>34</v>
+      <c r="BA5">
+        <v>0</v>
       </c>
       <c r="BB5" t="s">
         <v>34</v>
@@ -2822,13 +2837,16 @@
         <v>34</v>
       </c>
       <c r="BD5" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE5" t="s">
         <v>66</v>
       </c>
-      <c r="BE5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -2893,28 +2911,28 @@
         <v>34</v>
       </c>
       <c r="V6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W6" t="s">
         <v>64</v>
       </c>
       <c r="X6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y6" t="s">
         <v>65</v>
       </c>
       <c r="Z6" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA6" t="s">
         <v>42</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>101</v>
       </c>
       <c r="AB6" t="s">
         <v>102</v>
       </c>
       <c r="AC6" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD6" t="s">
         <v>34</v>
@@ -2923,70 +2941,70 @@
         <v>34</v>
       </c>
       <c r="AF6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG6" t="s">
         <v>35</v>
       </c>
-      <c r="AG6" s="3">
+      <c r="AH6" s="3">
         <v>60</v>
       </c>
-      <c r="AH6" s="3">
-        <v>30</v>
-      </c>
       <c r="AI6" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ6" s="3">
         <v>40</v>
       </c>
-      <c r="AJ6" s="3">
+      <c r="AK6" s="3">
         <v>1.4</v>
       </c>
-      <c r="AK6">
+      <c r="AL6">
         <v>5</v>
       </c>
-      <c r="AL6">
+      <c r="AM6">
         <v>21</v>
       </c>
-      <c r="AM6">
+      <c r="AN6">
         <v>125</v>
       </c>
-      <c r="AN6" s="3">
+      <c r="AO6" s="3">
         <v>7</v>
       </c>
-      <c r="AO6" s="3">
+      <c r="AP6" s="3">
         <v>2625</v>
       </c>
-      <c r="AP6" s="3">
+      <c r="AQ6" s="3">
         <v>0.36</v>
       </c>
-      <c r="AQ6" t="s">
+      <c r="AR6" t="s">
         <v>36</v>
       </c>
-      <c r="AR6" t="s">
+      <c r="AS6" t="s">
         <v>37</v>
       </c>
-      <c r="AS6" t="s">
+      <c r="AT6" t="s">
         <v>38</v>
       </c>
-      <c r="AT6" t="s">
+      <c r="AU6" t="s">
         <v>33</v>
       </c>
-      <c r="AU6" s="2">
+      <c r="AV6" s="2">
         <v>46192</v>
       </c>
-      <c r="AV6" s="2">
+      <c r="AW6" s="2">
         <v>46193</v>
       </c>
-      <c r="AW6" t="s">
-        <v>34</v>
-      </c>
       <c r="AX6" t="s">
         <v>34</v>
       </c>
-      <c r="AY6">
-        <v>0</v>
+      <c r="AY6" t="s">
+        <v>34</v>
       </c>
       <c r="AZ6">
         <v>0</v>
       </c>
-      <c r="BA6" t="s">
-        <v>34</v>
+      <c r="BA6">
+        <v>0</v>
       </c>
       <c r="BB6" t="s">
         <v>34</v>
@@ -2995,13 +3013,16 @@
         <v>34</v>
       </c>
       <c r="BD6" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE6" t="s">
         <v>66</v>
       </c>
-      <c r="BE6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -3066,28 +3087,28 @@
         <v>34</v>
       </c>
       <c r="V7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W7" t="s">
         <v>64</v>
       </c>
       <c r="X7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y7" t="s">
         <v>65</v>
       </c>
       <c r="Z7" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA7" t="s">
         <v>43</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>101</v>
       </c>
       <c r="AB7" t="s">
         <v>102</v>
       </c>
       <c r="AC7" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD7" t="s">
         <v>34</v>
@@ -3096,70 +3117,70 @@
         <v>34</v>
       </c>
       <c r="AF7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG7" t="s">
         <v>35</v>
       </c>
-      <c r="AG7" s="3">
+      <c r="AH7" s="3">
         <v>60</v>
       </c>
-      <c r="AH7" s="3">
-        <v>30</v>
-      </c>
       <c r="AI7" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ7" s="3">
         <v>40</v>
       </c>
-      <c r="AJ7" s="3">
+      <c r="AK7" s="3">
         <v>1.4</v>
       </c>
-      <c r="AK7">
+      <c r="AL7">
         <v>6</v>
       </c>
-      <c r="AL7">
+      <c r="AM7">
         <v>26</v>
       </c>
-      <c r="AM7">
+      <c r="AN7">
         <v>125</v>
       </c>
-      <c r="AN7" s="3">
+      <c r="AO7" s="3">
         <v>8.4</v>
       </c>
-      <c r="AO7" s="3">
+      <c r="AP7" s="3">
         <v>3250</v>
       </c>
-      <c r="AP7" s="3">
+      <c r="AQ7" s="3">
         <v>0.432</v>
       </c>
-      <c r="AQ7" t="s">
+      <c r="AR7" t="s">
         <v>36</v>
       </c>
-      <c r="AR7" t="s">
+      <c r="AS7" t="s">
         <v>37</v>
       </c>
-      <c r="AS7" t="s">
+      <c r="AT7" t="s">
         <v>38</v>
       </c>
-      <c r="AT7" t="s">
+      <c r="AU7" t="s">
         <v>33</v>
       </c>
-      <c r="AU7" s="2">
+      <c r="AV7" s="2">
         <v>46192</v>
       </c>
-      <c r="AV7" s="2">
+      <c r="AW7" s="2">
         <v>46193</v>
       </c>
-      <c r="AW7" t="s">
-        <v>34</v>
-      </c>
       <c r="AX7" t="s">
         <v>34</v>
       </c>
-      <c r="AY7">
-        <v>0</v>
+      <c r="AY7" t="s">
+        <v>34</v>
       </c>
       <c r="AZ7">
         <v>0</v>
       </c>
-      <c r="BA7" t="s">
-        <v>34</v>
+      <c r="BA7">
+        <v>0</v>
       </c>
       <c r="BB7" t="s">
         <v>34</v>
@@ -3168,13 +3189,16 @@
         <v>34</v>
       </c>
       <c r="BD7" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE7" t="s">
         <v>66</v>
       </c>
-      <c r="BE7" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="8" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -3239,28 +3263,28 @@
         <v>34</v>
       </c>
       <c r="V8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W8" t="s">
         <v>64</v>
       </c>
       <c r="X8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y8" t="s">
         <v>65</v>
       </c>
       <c r="Z8" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA8" t="s">
         <v>44</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>101</v>
       </c>
       <c r="AB8" t="s">
         <v>102</v>
       </c>
       <c r="AC8" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD8" t="s">
         <v>34</v>
@@ -3269,70 +3293,70 @@
         <v>34</v>
       </c>
       <c r="AF8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG8" t="s">
         <v>35</v>
       </c>
-      <c r="AG8" s="3">
+      <c r="AH8" s="3">
         <v>60</v>
       </c>
-      <c r="AH8" s="3">
-        <v>30</v>
-      </c>
       <c r="AI8" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ8" s="3">
         <v>40</v>
       </c>
-      <c r="AJ8" s="3">
+      <c r="AK8" s="3">
         <v>1.4</v>
       </c>
-      <c r="AK8">
+      <c r="AL8">
         <v>7</v>
       </c>
-      <c r="AL8">
+      <c r="AM8">
         <v>31</v>
       </c>
-      <c r="AM8">
+      <c r="AN8">
         <v>125</v>
       </c>
-      <c r="AN8" s="3">
+      <c r="AO8" s="3">
         <v>9.8</v>
       </c>
-      <c r="AO8" s="3">
+      <c r="AP8" s="3">
         <v>3875</v>
       </c>
-      <c r="AP8" s="3">
+      <c r="AQ8" s="3">
         <v>0.504</v>
       </c>
-      <c r="AQ8" t="s">
+      <c r="AR8" t="s">
         <v>36</v>
       </c>
-      <c r="AR8" t="s">
+      <c r="AS8" t="s">
         <v>37</v>
       </c>
-      <c r="AS8" t="s">
+      <c r="AT8" t="s">
         <v>38</v>
       </c>
-      <c r="AT8" t="s">
+      <c r="AU8" t="s">
         <v>33</v>
       </c>
-      <c r="AU8" s="2">
+      <c r="AV8" s="2">
         <v>46192</v>
       </c>
-      <c r="AV8" s="2">
+      <c r="AW8" s="2">
         <v>46193</v>
       </c>
-      <c r="AW8" t="s">
-        <v>34</v>
-      </c>
       <c r="AX8" t="s">
         <v>34</v>
       </c>
-      <c r="AY8">
-        <v>0</v>
+      <c r="AY8" t="s">
+        <v>34</v>
       </c>
       <c r="AZ8">
         <v>0</v>
       </c>
-      <c r="BA8" t="s">
-        <v>34</v>
+      <c r="BA8">
+        <v>0</v>
       </c>
       <c r="BB8" t="s">
         <v>34</v>
@@ -3341,13 +3365,16 @@
         <v>34</v>
       </c>
       <c r="BD8" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE8" t="s">
         <v>66</v>
       </c>
-      <c r="BE8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="BF8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -3412,28 +3439,28 @@
         <v>34</v>
       </c>
       <c r="V9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W9" t="s">
         <v>64</v>
       </c>
       <c r="X9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Y9" t="s">
         <v>65</v>
       </c>
       <c r="Z9" t="s">
+        <v>63</v>
+      </c>
+      <c r="AA9" t="s">
         <v>45</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>101</v>
       </c>
       <c r="AB9" t="s">
         <v>102</v>
       </c>
       <c r="AC9" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="AD9" t="s">
         <v>34</v>
@@ -3442,70 +3469,70 @@
         <v>34</v>
       </c>
       <c r="AF9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG9" t="s">
         <v>35</v>
       </c>
-      <c r="AG9" s="3">
+      <c r="AH9" s="3">
         <v>60</v>
       </c>
-      <c r="AH9" s="3">
-        <v>30</v>
-      </c>
       <c r="AI9" s="3">
+        <v>30</v>
+      </c>
+      <c r="AJ9" s="3">
         <v>40</v>
       </c>
-      <c r="AJ9" s="3">
+      <c r="AK9" s="3">
         <v>1.4</v>
       </c>
-      <c r="AK9">
+      <c r="AL9">
         <v>8</v>
       </c>
-      <c r="AL9">
+      <c r="AM9">
         <v>36</v>
       </c>
-      <c r="AM9">
-        <v>0</v>
-      </c>
-      <c r="AN9" s="3">
+      <c r="AN9">
+        <v>0</v>
+      </c>
+      <c r="AO9" s="3">
         <v>11.2</v>
       </c>
-      <c r="AO9" s="3">
-        <v>0</v>
-      </c>
       <c r="AP9" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ9" s="3">
         <v>0.576</v>
       </c>
-      <c r="AQ9" t="s">
+      <c r="AR9" t="s">
         <v>36</v>
       </c>
-      <c r="AR9" t="s">
+      <c r="AS9" t="s">
         <v>37</v>
       </c>
-      <c r="AS9" t="s">
+      <c r="AT9" t="s">
         <v>38</v>
       </c>
-      <c r="AT9" t="s">
+      <c r="AU9" t="s">
         <v>33</v>
       </c>
-      <c r="AU9" s="2">
+      <c r="AV9" s="2">
         <v>46192</v>
       </c>
-      <c r="AV9" s="2">
+      <c r="AW9" s="2">
         <v>46193</v>
       </c>
-      <c r="AW9" t="s">
-        <v>34</v>
-      </c>
       <c r="AX9" t="s">
         <v>34</v>
       </c>
-      <c r="AY9">
-        <v>0</v>
+      <c r="AY9" t="s">
+        <v>34</v>
       </c>
       <c r="AZ9">
         <v>0</v>
       </c>
-      <c r="BA9" t="s">
-        <v>34</v>
+      <c r="BA9">
+        <v>0</v>
       </c>
       <c r="BB9" t="s">
         <v>34</v>
@@ -3514,10 +3541,13 @@
         <v>34</v>
       </c>
       <c r="BD9" t="s">
+        <v>34</v>
+      </c>
+      <c r="BE9" t="s">
         <v>66</v>
       </c>
-      <c r="BE9" t="s">
-        <v>103</v>
+      <c r="BF9" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -3539,16 +3569,16 @@
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3570,7 +3600,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -3587,7 +3617,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -3604,7 +3634,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3621,7 +3651,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3638,7 +3668,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -3655,7 +3685,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -3672,7 +3702,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -3689,7 +3719,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -3706,7 +3736,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -3723,7 +3753,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -3740,7 +3770,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -3757,7 +3787,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -3774,7 +3804,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -3791,7 +3821,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -3808,7 +3838,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -3825,7 +3855,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -3842,12 +3872,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -3866,22 +3896,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
VBKREQ lines based on ASN carrier feed rather PO, missing sku with 0 units,extra SKU warning, latest PO carrier feed
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="131">
   <si>
     <t>PO_Number</t>
   </si>
@@ -297,6 +297,12 @@
     <t>Transport_Mode_Code</t>
   </si>
   <si>
+    <t>40452200458206</t>
+  </si>
+  <si>
+    <t>BD</t>
+  </si>
+  <si>
     <t>GB</t>
   </si>
   <si>
@@ -309,7 +315,19 @@
     <t>SCA_AFS_TEST_05</t>
   </si>
   <si>
+    <t>BLACK</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
     <t>30</t>
+  </si>
+  <si>
+    <t>2200003625899</t>
+  </si>
+  <si>
+    <t>M</t>
   </si>
   <si>
     <t>Weight_KG</t>
@@ -1393,7 +1411,7 @@
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
         <v>51</v>
@@ -1423,7 +1441,7 @@
         <v>31</v>
       </c>
       <c r="M2" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="N2" t="s">
         <v>55</v>
@@ -1450,13 +1468,13 @@
         <v>31</v>
       </c>
       <c r="V2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="W2" t="s">
         <v>57</v>
       </c>
       <c r="X2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Y2" t="s">
         <v>58</v>
@@ -1468,19 +1486,19 @@
         <v>32</v>
       </c>
       <c r="AB2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AC2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AD2" t="s">
         <v>31</v>
       </c>
       <c r="AE2" t="s">
-        <v>31</v>
+        <v>99</v>
       </c>
       <c r="AF2" t="s">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="AG2" t="s">
         <v>34</v>
@@ -1558,7 +1576,7 @@
         <v>59</v>
       </c>
       <c r="BF2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:58" x14ac:dyDescent="0.25">
@@ -1569,7 +1587,7 @@
         <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="D3" t="s">
         <v>51</v>
@@ -1599,7 +1617,7 @@
         <v>31</v>
       </c>
       <c r="M3" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="N3" t="s">
         <v>55</v>
@@ -1626,13 +1644,13 @@
         <v>31</v>
       </c>
       <c r="V3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="W3" t="s">
         <v>57</v>
       </c>
       <c r="X3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Y3" t="s">
         <v>58</v>
@@ -1644,19 +1662,19 @@
         <v>38</v>
       </c>
       <c r="AB3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AC3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AD3" t="s">
-        <v>31</v>
+        <v>102</v>
       </c>
       <c r="AE3" t="s">
-        <v>31</v>
+        <v>99</v>
       </c>
       <c r="AF3" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="AG3" t="s">
         <v>34</v>
@@ -1734,7 +1752,7 @@
         <v>59</v>
       </c>
       <c r="BF3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1756,16 +1774,16 @@
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1787,7 +1805,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1804,7 +1822,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1821,7 +1839,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1838,7 +1856,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1855,7 +1873,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1872,7 +1890,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1889,7 +1907,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1906,7 +1924,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1923,7 +1941,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1940,7 +1958,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1957,7 +1975,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1974,7 +1992,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1991,7 +2009,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -2008,7 +2026,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -2025,7 +2043,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -2042,7 +2060,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -2059,12 +2077,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2083,22 +2101,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rename fetch blob and add time taken
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="129">
   <si>
     <t>PO_Number</t>
   </si>
@@ -108,240 +108,240 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>500034227630</t>
+    <t>500034227292</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>148723499</t>
+    <t>123478460</t>
   </si>
   <si>
     <t>CFS</t>
   </si>
   <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>Flat</t>
+  </si>
+  <si>
+    <t>Delivery</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>140260044</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>orderId</t>
+  </si>
+  <si>
+    <t>supplierName</t>
+  </si>
+  <si>
+    <t>supplierId</t>
+  </si>
+  <si>
+    <t>factoryName</t>
+  </si>
+  <si>
+    <t>factoryId</t>
+  </si>
+  <si>
+    <t>factoryCity</t>
+  </si>
+  <si>
+    <t>factoryCountry</t>
+  </si>
+  <si>
+    <t>fcName</t>
+  </si>
+  <si>
+    <t>fcId</t>
+  </si>
+  <si>
+    <t>carrierId</t>
+  </si>
+  <si>
+    <t>loadingPortId</t>
+  </si>
+  <si>
+    <t>incoterms</t>
+  </si>
+  <si>
+    <t>Tudorknight Limited (OB)</t>
+  </si>
+  <si>
+    <t>1100004812</t>
+  </si>
+  <si>
+    <t>Dummy Factory</t>
+  </si>
+  <si>
+    <t>9999</t>
+  </si>
+  <si>
+    <t>FC01 Barnsley</t>
+  </si>
+  <si>
+    <t>FC01</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>TURIS</t>
+  </si>
+  <si>
+    <t>FOB</t>
+  </si>
+  <si>
+    <t>documentId</t>
+  </si>
+  <si>
+    <t>receivedDate</t>
+  </si>
+  <si>
+    <t>sku</t>
+  </si>
+  <si>
+    <t>receivedQty</t>
+  </si>
+  <si>
+    <t>shipmentRef</t>
+  </si>
+  <si>
+    <t>Booking_Ref</t>
+  </si>
+  <si>
+    <t>Supplier_Name</t>
+  </si>
+  <si>
+    <t>Supplier_ID</t>
+  </si>
+  <si>
+    <t>Factory_Name</t>
+  </si>
+  <si>
+    <t>Factory_ID</t>
+  </si>
+  <si>
+    <t>Factory_Street1</t>
+  </si>
+  <si>
+    <t>Factory_Street2</t>
+  </si>
+  <si>
+    <t>Factory_Street3</t>
+  </si>
+  <si>
+    <t>Factory_City</t>
+  </si>
+  <si>
+    <t>Factory_PostalCd</t>
+  </si>
+  <si>
+    <t>Factory_CountryCd</t>
+  </si>
+  <si>
+    <t>FC_Name</t>
+  </si>
+  <si>
+    <t>FC_ID</t>
+  </si>
+  <si>
+    <t>FC_Street1</t>
+  </si>
+  <si>
+    <t>FC_Street2</t>
+  </si>
+  <si>
+    <t>FC_Street3</t>
+  </si>
+  <si>
+    <t>FC_City</t>
+  </si>
+  <si>
+    <t>FC_StateProvinceCd</t>
+  </si>
+  <si>
+    <t>FC_PostalCd</t>
+  </si>
+  <si>
+    <t>FC_CountryCd</t>
+  </si>
+  <si>
+    <t>Carrier_ID</t>
+  </si>
+  <si>
+    <t>Carrier_Name</t>
+  </si>
+  <si>
+    <t>Loading_Port_LOCODE</t>
+  </si>
+  <si>
+    <t>F1_ID</t>
+  </si>
+  <si>
+    <t>Product_Style</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Incoterms</t>
+  </si>
+  <si>
+    <t>Transport_Mode_Code</t>
+  </si>
+  <si>
+    <t>45870000002757</t>
+  </si>
+  <si>
+    <t>BD</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>European Nom Carrier</t>
+  </si>
+  <si>
+    <t>123478454</t>
+  </si>
+  <si>
+    <t>HONEY REV</t>
+  </si>
+  <si>
+    <t>BLACK</t>
+  </si>
+  <si>
+    <t>UK 10</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Weight_KG</t>
+  </si>
+  <si>
+    <t>Length_cm</t>
+  </si>
+  <si>
+    <t>Width_cm</t>
+  </si>
+  <si>
+    <t>Height_cm</t>
+  </si>
+  <si>
     <t>BDCM1</t>
   </si>
   <si>
-    <t>Flat</t>
-  </si>
-  <si>
-    <t>Delivery</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>148723500</t>
-  </si>
-  <si>
-    <t>orderId</t>
-  </si>
-  <si>
-    <t>supplierName</t>
-  </si>
-  <si>
-    <t>supplierId</t>
-  </si>
-  <si>
-    <t>factoryName</t>
-  </si>
-  <si>
-    <t>factoryId</t>
-  </si>
-  <si>
-    <t>factoryCity</t>
-  </si>
-  <si>
-    <t>factoryCountry</t>
-  </si>
-  <si>
-    <t>fcName</t>
-  </si>
-  <si>
-    <t>fcId</t>
-  </si>
-  <si>
-    <t>carrierId</t>
-  </si>
-  <si>
-    <t>loadingPortId</t>
-  </si>
-  <si>
-    <t>incoterms</t>
-  </si>
-  <si>
-    <t>Scalpers AFS (UK)</t>
-  </si>
-  <si>
-    <t>2002680002</t>
-  </si>
-  <si>
-    <t>Dummy Factory</t>
-  </si>
-  <si>
-    <t>9999</t>
-  </si>
-  <si>
-    <t>FC01 Barnsley</t>
-  </si>
-  <si>
-    <t>FC01</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>SPVAL</t>
-  </si>
-  <si>
-    <t>FOB</t>
-  </si>
-  <si>
-    <t>documentId</t>
-  </si>
-  <si>
-    <t>receivedDate</t>
-  </si>
-  <si>
-    <t>sku</t>
-  </si>
-  <si>
-    <t>receivedQty</t>
-  </si>
-  <si>
-    <t>shipmentRef</t>
-  </si>
-  <si>
-    <t>Booking_Ref</t>
-  </si>
-  <si>
-    <t>Supplier_Name</t>
-  </si>
-  <si>
-    <t>Supplier_ID</t>
-  </si>
-  <si>
-    <t>Factory_Name</t>
-  </si>
-  <si>
-    <t>Factory_ID</t>
-  </si>
-  <si>
-    <t>Factory_Street1</t>
-  </si>
-  <si>
-    <t>Factory_Street2</t>
-  </si>
-  <si>
-    <t>Factory_Street3</t>
-  </si>
-  <si>
-    <t>Factory_City</t>
-  </si>
-  <si>
-    <t>Factory_PostalCd</t>
-  </si>
-  <si>
-    <t>Factory_CountryCd</t>
-  </si>
-  <si>
-    <t>FC_Name</t>
-  </si>
-  <si>
-    <t>FC_ID</t>
-  </si>
-  <si>
-    <t>FC_Street1</t>
-  </si>
-  <si>
-    <t>FC_Street2</t>
-  </si>
-  <si>
-    <t>FC_Street3</t>
-  </si>
-  <si>
-    <t>FC_City</t>
-  </si>
-  <si>
-    <t>FC_StateProvinceCd</t>
-  </si>
-  <si>
-    <t>FC_PostalCd</t>
-  </si>
-  <si>
-    <t>FC_CountryCd</t>
-  </si>
-  <si>
-    <t>Carrier_ID</t>
-  </si>
-  <si>
-    <t>Carrier_Name</t>
-  </si>
-  <si>
-    <t>Loading_Port_LOCODE</t>
-  </si>
-  <si>
-    <t>F1_ID</t>
-  </si>
-  <si>
-    <t>Product_Style</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Incoterms</t>
-  </si>
-  <si>
-    <t>Transport_Mode_Code</t>
-  </si>
-  <si>
-    <t>40452200458206</t>
-  </si>
-  <si>
-    <t>BD</t>
-  </si>
-  <si>
-    <t>GB</t>
-  </si>
-  <si>
-    <t>European Nom Carrier</t>
-  </si>
-  <si>
-    <t>148723498</t>
-  </si>
-  <si>
-    <t>SCA_AFS_TEST_05</t>
-  </si>
-  <si>
-    <t>BLACK</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>2200003625899</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>Weight_KG</t>
-  </si>
-  <si>
-    <t>Length_cm</t>
-  </si>
-  <si>
-    <t>Width_cm</t>
-  </si>
-  <si>
-    <t>Height_cm</t>
-  </si>
-  <si>
     <t>BDCM3</t>
   </si>
   <si>
@@ -349,12 +349,6 @@
   </si>
   <si>
     <t>Cartons</t>
-  </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t>A2</t>
   </si>
   <si>
     <t>A3</t>
@@ -913,10 +907,10 @@
         <v>32</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" s="2">
         <v>46192</v>
@@ -940,25 +934,25 @@
         <v>34</v>
       </c>
       <c r="M2">
-        <v>60</v>
+        <v>59.5</v>
       </c>
       <c r="N2">
-        <v>30</v>
+        <v>28.5</v>
       </c>
       <c r="O2">
-        <v>40</v>
+        <v>32.5</v>
       </c>
       <c r="P2">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="Q2">
-        <v>1.4</v>
+        <v>11</v>
       </c>
       <c r="R2">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="S2">
-        <v>0.072</v>
+        <v>0.606230625</v>
       </c>
       <c r="T2">
         <v>10</v>
@@ -1005,10 +999,10 @@
         <v>38</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F3" s="2">
         <v>46192</v>
@@ -1029,31 +1023,31 @@
         <v>31</v>
       </c>
       <c r="L3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="M3">
-        <v>60</v>
+        <v>59.5</v>
       </c>
       <c r="N3">
-        <v>30</v>
+        <v>28.5</v>
       </c>
       <c r="O3">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="P3">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="Q3">
-        <v>1.4</v>
+        <v>12</v>
       </c>
       <c r="R3">
-        <v>10</v>
+        <v>1440</v>
       </c>
       <c r="S3">
-        <v>0.072</v>
+        <v>0.7630874999999999</v>
       </c>
       <c r="T3">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="U3" t="s">
         <v>35</v>
@@ -1102,40 +1096,40 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1143,16 +1137,16 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F2" t="s">
         <v>31</v>
@@ -1161,19 +1155,19 @@
         <v>31</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="L2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1192,25 +1186,25 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1221,7 +1215,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BF3"/>
+  <dimension ref="A1:BF2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="58" width="22" customWidth="1"/>
@@ -1229,7 +1223,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1238,82 +1232,82 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>8</v>
@@ -1397,10 +1391,10 @@
         <v>22</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:58" x14ac:dyDescent="0.25">
@@ -1411,19 +1405,19 @@
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H2" t="s">
         <v>31</v>
@@ -1441,13 +1435,13 @@
         <v>31</v>
       </c>
       <c r="M2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="N2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P2" t="s">
         <v>31</v>
@@ -1468,70 +1462,70 @@
         <v>31</v>
       </c>
       <c r="V2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="W2" t="s">
+        <v>58</v>
+      </c>
+      <c r="X2" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z2" t="s">
         <v>57</v>
-      </c>
-      <c r="X2" t="s">
-        <v>96</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>56</v>
       </c>
       <c r="AA2" t="s">
         <v>32</v>
       </c>
       <c r="AB2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AC2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AD2" t="s">
         <v>31</v>
       </c>
       <c r="AE2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AG2" t="s">
         <v>34</v>
       </c>
       <c r="AH2" s="3">
-        <v>60</v>
+        <v>59.5</v>
       </c>
       <c r="AI2" s="3">
-        <v>30</v>
+        <v>28.5</v>
       </c>
       <c r="AJ2" s="3">
-        <v>40</v>
+        <v>32.5</v>
       </c>
       <c r="AK2" s="3">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="AL2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AM2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN2">
         <v>10</v>
       </c>
       <c r="AO2" s="3">
-        <v>1.4</v>
+        <v>11</v>
       </c>
       <c r="AP2" s="3">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="AQ2" s="3">
-        <v>0.072</v>
+        <v>0.6062</v>
       </c>
       <c r="AR2" t="s">
         <v>35</v>
@@ -1573,186 +1567,10 @@
         <v>31</v>
       </c>
       <c r="BE2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="BF2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>93</v>
-      </c>
-      <c r="D3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3" t="s">
-        <v>94</v>
-      </c>
-      <c r="N3" t="s">
-        <v>55</v>
-      </c>
-      <c r="O3" t="s">
-        <v>56</v>
-      </c>
-      <c r="P3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R3" t="s">
-        <v>31</v>
-      </c>
-      <c r="S3" t="s">
-        <v>31</v>
-      </c>
-      <c r="T3" t="s">
-        <v>31</v>
-      </c>
-      <c r="U3" t="s">
-        <v>31</v>
-      </c>
-      <c r="V3" t="s">
-        <v>95</v>
-      </c>
-      <c r="W3" t="s">
-        <v>57</v>
-      </c>
-      <c r="X3" t="s">
-        <v>96</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>97</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AD3" t="s">
         <v>102</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>99</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>103</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>34</v>
-      </c>
-      <c r="AH3" s="3">
-        <v>60</v>
-      </c>
-      <c r="AI3" s="3">
-        <v>30</v>
-      </c>
-      <c r="AJ3" s="3">
-        <v>40</v>
-      </c>
-      <c r="AK3" s="3">
-        <v>1.4</v>
-      </c>
-      <c r="AL3">
-        <v>1</v>
-      </c>
-      <c r="AM3">
-        <v>1</v>
-      </c>
-      <c r="AN3">
-        <v>10</v>
-      </c>
-      <c r="AO3" s="3">
-        <v>1.4</v>
-      </c>
-      <c r="AP3" s="3">
-        <v>10</v>
-      </c>
-      <c r="AQ3" s="3">
-        <v>0.072</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>36</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>37</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>33</v>
-      </c>
-      <c r="AV3" s="2">
-        <v>46192</v>
-      </c>
-      <c r="AW3" s="2">
-        <v>46193</v>
-      </c>
-      <c r="AX3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AY3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AZ3">
-        <v>0</v>
-      </c>
-      <c r="BA3">
-        <v>0</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>31</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>31</v>
-      </c>
-      <c r="BD3" t="s">
-        <v>31</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>59</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1774,21 +1592,21 @@
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>107</v>
       </c>
       <c r="B2">
         <v>1.4</v>
@@ -1856,7 +1674,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1873,7 +1691,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1890,7 +1708,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1907,7 +1725,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1924,7 +1742,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1941,7 +1759,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1958,7 +1776,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1975,7 +1793,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1992,7 +1810,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -2009,7 +1827,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -2026,7 +1844,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -2043,7 +1861,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -2060,7 +1878,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -2077,12 +1895,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2101,22 +1919,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Table mapping on blob result
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="144">
   <si>
     <t>PO_Number</t>
   </si>
@@ -201,19 +201,79 @@
     <t>FOB</t>
   </si>
   <si>
-    <t>documentId</t>
-  </si>
-  <si>
-    <t>receivedDate</t>
+    <t>filename</t>
+  </si>
+  <si>
+    <t>blobPath</t>
+  </si>
+  <si>
+    <t>asnId</t>
+  </si>
+  <si>
+    <t>poId</t>
+  </si>
+  <si>
+    <t>shipDate</t>
+  </si>
+  <si>
+    <t>supplier</t>
   </si>
   <si>
     <t>sku</t>
   </si>
   <si>
-    <t>receivedQty</t>
-  </si>
-  <si>
-    <t>shipmentRef</t>
+    <t>ean</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>colour</t>
+  </si>
+  <si>
+    <t>style</t>
+  </si>
+  <si>
+    <t>packFormat</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>ASOS_20260519_1448_DavisTurner_0000.xml</t>
+  </si>
+  <si>
+    <t>ASNInDavisTurner/2026/05/19/ASOS_20260519_1448_DavisTurner_0000.xml</t>
+  </si>
+  <si>
+    <t>45870000002757</t>
+  </si>
+  <si>
+    <t>2026-06-17</t>
+  </si>
+  <si>
+    <t>Sku Publish1746626784</t>
+  </si>
+  <si>
+    <t>UK 10</t>
+  </si>
+  <si>
+    <t>BLACK</t>
+  </si>
+  <si>
+    <t>123478454</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>BD</t>
   </si>
   <si>
     <t>Booking_Ref</t>
@@ -300,28 +360,13 @@
     <t>Transport_Mode_Code</t>
   </si>
   <si>
-    <t>45870000002757</t>
-  </si>
-  <si>
-    <t>BD</t>
-  </si>
-  <si>
     <t>GB</t>
   </si>
   <si>
     <t>European Nom Carrier</t>
   </si>
   <si>
-    <t>123478454</t>
-  </si>
-  <si>
     <t>HONEY REV</t>
-  </si>
-  <si>
-    <t>BLACK</t>
-  </si>
-  <si>
-    <t>UK 10</t>
   </si>
   <si>
     <t>30</t>
@@ -1178,33 +1223,110 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="7" width="22" customWidth="1"/>
+    <col min="1" max="16" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" t="s">
+        <v>82</v>
+      </c>
+      <c r="M2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N2" t="s">
+        <v>84</v>
+      </c>
+      <c r="O2" t="s">
+        <v>85</v>
+      </c>
+      <c r="P2">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1223,7 +1345,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1232,82 +1354,82 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>8</v>
@@ -1391,10 +1513,10 @@
         <v>22</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:58" x14ac:dyDescent="0.25">
@@ -1405,7 +1527,7 @@
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
         <v>52</v>
@@ -1435,7 +1557,7 @@
         <v>31</v>
       </c>
       <c r="M2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="N2" t="s">
         <v>56</v>
@@ -1462,13 +1584,13 @@
         <v>31</v>
       </c>
       <c r="V2" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="W2" t="s">
         <v>58</v>
       </c>
       <c r="X2" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="Y2" t="s">
         <v>59</v>
@@ -1480,19 +1602,19 @@
         <v>32</v>
       </c>
       <c r="AB2" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="AC2" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="AD2" t="s">
         <v>31</v>
       </c>
       <c r="AE2" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AF2" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="AG2" t="s">
         <v>34</v>
@@ -1570,7 +1692,7 @@
         <v>60</v>
       </c>
       <c r="BF2" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1592,21 +1714,21 @@
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B2">
         <v>1.4</v>
@@ -1623,7 +1745,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1640,7 +1762,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1657,7 +1779,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1708,7 +1830,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1725,7 +1847,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1742,7 +1864,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1759,7 +1881,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1776,7 +1898,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1793,7 +1915,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1810,7 +1932,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1827,7 +1949,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1844,7 +1966,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1861,7 +1983,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1878,7 +2000,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -1895,12 +2017,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1919,22 +2041,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
log fix,multiple vbkreqs,Cols reshuffle on supplier book,added calender
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="133">
   <si>
     <t>PO_Number</t>
   </si>
@@ -242,157 +242,103 @@
     <t>quantity</t>
   </si>
   <si>
-    <t>ASOS_20260613_0212_DavisTurner_0010.xml</t>
-  </si>
-  <si>
-    <t>ASNInDavisTurner/2026/06/13/ASOS_20260613_0212_DavisTurner_0010.xml</t>
-  </si>
-  <si>
-    <t>45870000003922</t>
+    <t>Booking_Ref</t>
+  </si>
+  <si>
+    <t>Supplier_Name</t>
+  </si>
+  <si>
+    <t>Supplier_ID</t>
+  </si>
+  <si>
+    <t>Factory_Street3</t>
+  </si>
+  <si>
+    <t>Country_Of_Origin</t>
+  </si>
+  <si>
+    <t>FC_ID</t>
+  </si>
+  <si>
+    <t>FC_Name</t>
+  </si>
+  <si>
+    <t>FC_Street1</t>
+  </si>
+  <si>
+    <t>FC_Street2</t>
+  </si>
+  <si>
+    <t>FC_Street3</t>
+  </si>
+  <si>
+    <t>FC_City</t>
+  </si>
+  <si>
+    <t>FC_StateProvinceCd</t>
+  </si>
+  <si>
+    <t>FC_PostalCd</t>
+  </si>
+  <si>
+    <t>FC_CountryCd</t>
+  </si>
+  <si>
+    <t>Carrier_ID</t>
+  </si>
+  <si>
+    <t>Carrier_Name</t>
+  </si>
+  <si>
+    <t>Loading_Port_LOCODE</t>
+  </si>
+  <si>
+    <t>F1_ID</t>
+  </si>
+  <si>
+    <t>Product_Style</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Incoterms</t>
+  </si>
+  <si>
+    <t>Transport_Mode_Code</t>
   </si>
   <si>
     <t>FC01</t>
   </si>
   <si>
-    <t>2026-07-11</t>
-  </si>
-  <si>
-    <t>Tudorknight Limited (OB)</t>
-  </si>
-  <si>
-    <t>1100004812</t>
-  </si>
-  <si>
-    <t>TURKEY ISTANBUL</t>
-  </si>
-  <si>
-    <t>FOB</t>
+    <t>ASOS Barnsley</t>
+  </si>
+  <si>
+    <t>Langthwaite Grange Industrial Estate</t>
+  </si>
+  <si>
+    <t>South Kirkby</t>
+  </si>
+  <si>
+    <t>WF9 3NR</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>3</t>
   </si>
   <si>
     <t>123478465</t>
   </si>
   <si>
-    <t>Sku Publish1746626784</t>
-  </si>
-  <si>
-    <t>UK 6</t>
-  </si>
-  <si>
-    <t>BLACK</t>
-  </si>
-  <si>
-    <t>123478454</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>BD</t>
+    <t>30</t>
   </si>
   <si>
     <t>123478466</t>
   </si>
   <si>
-    <t>UK 8</t>
-  </si>
-  <si>
     <t>123478467</t>
-  </si>
-  <si>
-    <t>UK 4</t>
-  </si>
-  <si>
-    <t>45870000003923</t>
-  </si>
-  <si>
-    <t>Booking_Ref</t>
-  </si>
-  <si>
-    <t>Supplier_Name</t>
-  </si>
-  <si>
-    <t>Supplier_ID</t>
-  </si>
-  <si>
-    <t>Factory_Street3</t>
-  </si>
-  <si>
-    <t>Country_Of_Origin</t>
-  </si>
-  <si>
-    <t>FC_ID</t>
-  </si>
-  <si>
-    <t>FC_Name</t>
-  </si>
-  <si>
-    <t>FC_Street1</t>
-  </si>
-  <si>
-    <t>FC_Street2</t>
-  </si>
-  <si>
-    <t>FC_Street3</t>
-  </si>
-  <si>
-    <t>FC_City</t>
-  </si>
-  <si>
-    <t>FC_StateProvinceCd</t>
-  </si>
-  <si>
-    <t>FC_PostalCd</t>
-  </si>
-  <si>
-    <t>FC_CountryCd</t>
-  </si>
-  <si>
-    <t>Carrier_ID</t>
-  </si>
-  <si>
-    <t>Carrier_Name</t>
-  </si>
-  <si>
-    <t>Loading_Port_LOCODE</t>
-  </si>
-  <si>
-    <t>F1_ID</t>
-  </si>
-  <si>
-    <t>Product_Style</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Incoterms</t>
-  </si>
-  <si>
-    <t>Transport_Mode_Code</t>
-  </si>
-  <si>
-    <t>ASOS Barnsley</t>
-  </si>
-  <si>
-    <t>Langthwaite Grange Industrial Estate</t>
-  </si>
-  <si>
-    <t>South Kirkby</t>
-  </si>
-  <si>
-    <t>WF9 3NR</t>
-  </si>
-  <si>
-    <t>GB</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>SKU from carrier feed — not found in supplier template</t>
   </si>
   <si>
     <t>Weight_KG</t>
@@ -487,7 +433,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,11 +450,6 @@
         <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -522,14 +463,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1579,7 +1519,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="19" width="22" customWidth="1"/>
@@ -1644,360 +1584,6 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G2" t="s">
-        <v>80</v>
-      </c>
-      <c r="H2" t="s">
-        <v>81</v>
-      </c>
-      <c r="I2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J2" t="s">
-        <v>83</v>
-      </c>
-      <c r="K2" t="s">
-        <v>84</v>
-      </c>
-      <c r="L2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" t="s">
-        <v>85</v>
-      </c>
-      <c r="N2" t="s">
-        <v>86</v>
-      </c>
-      <c r="O2" t="s">
-        <v>87</v>
-      </c>
-      <c r="P2" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>89</v>
-      </c>
-      <c r="R2" t="s">
-        <v>90</v>
-      </c>
-      <c r="S2">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" t="s">
-        <v>79</v>
-      </c>
-      <c r="G3" t="s">
-        <v>80</v>
-      </c>
-      <c r="H3" t="s">
-        <v>81</v>
-      </c>
-      <c r="I3" t="s">
-        <v>82</v>
-      </c>
-      <c r="J3" t="s">
-        <v>83</v>
-      </c>
-      <c r="K3" t="s">
-        <v>91</v>
-      </c>
-      <c r="L3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>85</v>
-      </c>
-      <c r="N3" t="s">
-        <v>92</v>
-      </c>
-      <c r="O3" t="s">
-        <v>87</v>
-      </c>
-      <c r="P3" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>89</v>
-      </c>
-      <c r="R3" t="s">
-        <v>90</v>
-      </c>
-      <c r="S3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G4" t="s">
-        <v>80</v>
-      </c>
-      <c r="H4" t="s">
-        <v>81</v>
-      </c>
-      <c r="I4" t="s">
-        <v>82</v>
-      </c>
-      <c r="J4" t="s">
-        <v>83</v>
-      </c>
-      <c r="K4" t="s">
-        <v>93</v>
-      </c>
-      <c r="L4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M4" t="s">
-        <v>85</v>
-      </c>
-      <c r="N4" t="s">
-        <v>94</v>
-      </c>
-      <c r="O4" t="s">
-        <v>87</v>
-      </c>
-      <c r="P4" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>89</v>
-      </c>
-      <c r="R4" t="s">
-        <v>90</v>
-      </c>
-      <c r="S4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G5" t="s">
-        <v>80</v>
-      </c>
-      <c r="H5" t="s">
-        <v>81</v>
-      </c>
-      <c r="I5" t="s">
-        <v>82</v>
-      </c>
-      <c r="J5" t="s">
-        <v>83</v>
-      </c>
-      <c r="K5" t="s">
-        <v>84</v>
-      </c>
-      <c r="L5" t="s">
-        <v>39</v>
-      </c>
-      <c r="M5" t="s">
-        <v>85</v>
-      </c>
-      <c r="N5" t="s">
-        <v>86</v>
-      </c>
-      <c r="O5" t="s">
-        <v>87</v>
-      </c>
-      <c r="P5" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>89</v>
-      </c>
-      <c r="R5" t="s">
-        <v>90</v>
-      </c>
-      <c r="S5">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" t="s">
-        <v>95</v>
-      </c>
-      <c r="D6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" t="s">
-        <v>80</v>
-      </c>
-      <c r="H6" t="s">
-        <v>81</v>
-      </c>
-      <c r="I6" t="s">
-        <v>82</v>
-      </c>
-      <c r="J6" t="s">
-        <v>83</v>
-      </c>
-      <c r="K6" t="s">
-        <v>91</v>
-      </c>
-      <c r="L6" t="s">
-        <v>39</v>
-      </c>
-      <c r="M6" t="s">
-        <v>85</v>
-      </c>
-      <c r="N6" t="s">
-        <v>92</v>
-      </c>
-      <c r="O6" t="s">
-        <v>87</v>
-      </c>
-      <c r="P6" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>89</v>
-      </c>
-      <c r="R6" t="s">
-        <v>90</v>
-      </c>
-      <c r="S6">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" t="s">
-        <v>95</v>
-      </c>
-      <c r="D7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G7" t="s">
-        <v>80</v>
-      </c>
-      <c r="H7" t="s">
-        <v>81</v>
-      </c>
-      <c r="I7" t="s">
-        <v>82</v>
-      </c>
-      <c r="J7" t="s">
-        <v>83</v>
-      </c>
-      <c r="K7" t="s">
-        <v>93</v>
-      </c>
-      <c r="L7" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" t="s">
-        <v>85</v>
-      </c>
-      <c r="N7" t="s">
-        <v>94</v>
-      </c>
-      <c r="O7" t="s">
-        <v>87</v>
-      </c>
-      <c r="P7" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>89</v>
-      </c>
-      <c r="R7" t="s">
-        <v>90</v>
-      </c>
-      <c r="S7">
-        <v>100</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2006,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BH7"/>
+  <dimension ref="A1:BH6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="60" width="22" customWidth="1"/>
@@ -2014,7 +1600,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2023,10 +1609,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>9</v>
@@ -2041,7 +1627,7 @@
         <v>12</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>13</v>
@@ -2053,55 +1639,55 @@
         <v>15</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="AE1" s="1" t="s">
         <v>16</v>
@@ -2188,10 +1774,10 @@
         <v>30</v>
       </c>
       <c r="BG1" s="1" t="s">
-        <v>116</v>
+        <v>95</v>
       </c>
       <c r="BH1" s="1" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:60" x14ac:dyDescent="0.25">
@@ -2202,13 +1788,13 @@
         <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="F2" t="s">
         <v>42</v>
@@ -2235,16 +1821,16 @@
         <v>46</v>
       </c>
       <c r="N2" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="O2" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="P2" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="Q2" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="R2" t="s">
         <v>39</v>
@@ -2253,46 +1839,46 @@
         <v>39</v>
       </c>
       <c r="T2" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="U2" t="s">
         <v>39</v>
       </c>
       <c r="V2" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="W2" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="X2" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="Y2" t="s">
         <v>39</v>
       </c>
       <c r="Z2" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="AA2" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="AB2" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="AC2" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="AD2" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="AE2" t="s">
         <v>39</v>
       </c>
       <c r="AF2" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="AG2" t="s">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="AH2" t="s">
         <v>47</v>
@@ -2370,10 +1956,10 @@
         <v>39</v>
       </c>
       <c r="BG2" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="BH2" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:60" x14ac:dyDescent="0.25">
@@ -2384,13 +1970,13 @@
         <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
         <v>42</v>
@@ -2417,16 +2003,16 @@
         <v>46</v>
       </c>
       <c r="N3" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="O3" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="P3" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="Q3" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="R3" t="s">
         <v>39</v>
@@ -2435,46 +2021,46 @@
         <v>39</v>
       </c>
       <c r="T3" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="U3" t="s">
         <v>39</v>
       </c>
       <c r="V3" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="W3" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="X3" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="Y3" t="s">
         <v>39</v>
       </c>
       <c r="Z3" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="AA3" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="AB3" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="AC3" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="AD3" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="AE3" t="s">
         <v>39</v>
       </c>
       <c r="AF3" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="AG3" t="s">
-        <v>92</v>
+        <v>39</v>
       </c>
       <c r="AH3" t="s">
         <v>51</v>
@@ -2552,10 +2138,10 @@
         <v>39</v>
       </c>
       <c r="BG3" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="BH3" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:60" x14ac:dyDescent="0.25">
@@ -2566,13 +2152,13 @@
         <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="F4" t="s">
         <v>42</v>
@@ -2599,16 +2185,16 @@
         <v>46</v>
       </c>
       <c r="N4" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="O4" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="P4" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="Q4" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="R4" t="s">
         <v>39</v>
@@ -2617,46 +2203,46 @@
         <v>39</v>
       </c>
       <c r="T4" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="U4" t="s">
         <v>39</v>
       </c>
       <c r="V4" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="W4" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="X4" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="Y4" t="s">
         <v>39</v>
       </c>
       <c r="Z4" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="AA4" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="AB4" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="AC4" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="AD4" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="AE4" t="s">
         <v>39</v>
       </c>
       <c r="AF4" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="AG4" t="s">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="AH4" t="s">
         <v>47</v>
@@ -2734,10 +2320,10 @@
         <v>39</v>
       </c>
       <c r="BG4" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="BH4" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:60" x14ac:dyDescent="0.25">
@@ -2748,13 +2334,13 @@
         <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
         <v>42</v>
@@ -2781,16 +2367,16 @@
         <v>46</v>
       </c>
       <c r="N5" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="O5" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="P5" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="Q5" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="R5" t="s">
         <v>39</v>
@@ -2799,46 +2385,46 @@
         <v>39</v>
       </c>
       <c r="T5" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="U5" t="s">
         <v>39</v>
       </c>
       <c r="V5" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="W5" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="X5" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="Y5" t="s">
         <v>39</v>
       </c>
       <c r="Z5" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="AA5" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="AB5" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="AC5" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="AD5" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="AE5" t="s">
         <v>39</v>
       </c>
       <c r="AF5" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="AG5" t="s">
-        <v>92</v>
+        <v>39</v>
       </c>
       <c r="AH5" t="s">
         <v>51</v>
@@ -2916,10 +2502,10 @@
         <v>39</v>
       </c>
       <c r="BG5" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="BH5" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:60" x14ac:dyDescent="0.25">
@@ -2930,13 +2516,13 @@
         <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
         <v>42</v>
@@ -2963,16 +2549,16 @@
         <v>46</v>
       </c>
       <c r="N6" t="s">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="O6" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="P6" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="Q6" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="R6" t="s">
         <v>39</v>
@@ -2981,46 +2567,46 @@
         <v>39</v>
       </c>
       <c r="T6" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="U6" t="s">
         <v>39</v>
       </c>
       <c r="V6" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="W6" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="X6" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="Y6" t="s">
         <v>39</v>
       </c>
       <c r="Z6" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="AA6" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="AB6" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="AC6" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="AD6" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="AE6" t="s">
         <v>39</v>
       </c>
       <c r="AF6" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="AG6" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="AH6" t="s">
         <v>55</v>
@@ -3098,192 +2684,10 @@
         <v>39</v>
       </c>
       <c r="BG6" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="BH6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="O7" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="P7" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q7" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="R7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="S7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T7" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="U7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="V7" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="W7" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="X7" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="Y7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z7" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA7" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB7" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="AC7" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="AD7" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="AE7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AF7" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="AG7" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="AH7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="AI7" s="3">
-        <v>60</v>
-      </c>
-      <c r="AJ7" s="3">
-        <v>30</v>
-      </c>
-      <c r="AK7" s="3">
-        <v>40</v>
-      </c>
-      <c r="AL7" s="3">
-        <v>1.4</v>
-      </c>
-      <c r="AM7" s="4">
-        <v>0</v>
-      </c>
-      <c r="AN7" s="4">
-        <v>0</v>
-      </c>
-      <c r="AO7" s="4">
-        <v>0</v>
-      </c>
-      <c r="AP7" s="3">
-        <v>0</v>
-      </c>
-      <c r="AQ7" s="3">
-        <v>0</v>
-      </c>
-      <c r="AR7" s="3">
-        <v>0</v>
-      </c>
-      <c r="AS7" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AT7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="AU7" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="AV7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AW7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AX7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AY7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AZ7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BA7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BB7" s="4">
-        <v>0</v>
-      </c>
-      <c r="BC7" s="4">
-        <v>0</v>
-      </c>
-      <c r="BD7" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="BE7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BF7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BG7" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="BH7" s="4" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -3305,16 +2709,16 @@
         <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3370,7 +2774,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3387,7 +2791,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3404,7 +2808,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -3421,7 +2825,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -3438,7 +2842,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -3455,7 +2859,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -3472,7 +2876,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -3489,7 +2893,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -3506,7 +2910,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -3523,7 +2927,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -3540,7 +2944,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -3557,7 +2961,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -3574,7 +2978,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -3591,7 +2995,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -3608,12 +3012,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3632,22 +3036,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Supplier template sheet name change, instruction, UI modification,pack  to bulk flat,ASN ref on result
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="145">
   <si>
     <t>PO_Number</t>
   </si>
@@ -131,7 +131,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>500034236926</t>
+    <t>500034236928</t>
   </si>
   <si>
     <t/>
@@ -152,7 +152,7 @@
     <t>BDCM1</t>
   </si>
   <si>
-    <t>Flat</t>
+    <t>Bulk Flat</t>
   </si>
   <si>
     <t>Delivery</t>
@@ -218,13 +218,13 @@
     <t>quantity</t>
   </si>
   <si>
-    <t>ASOS_20260617_0732_DavisTurner_0000.xml</t>
-  </si>
-  <si>
-    <t>ASNInDavisTurner/2026/06/17/ASOS_20260617_0732_DavisTurner_0000.xml</t>
-  </si>
-  <si>
-    <t>49870000004091</t>
+    <t>ASOS_20260617_0740_DavisTurner_0002.xml</t>
+  </si>
+  <si>
+    <t>ASNInDavisTurner/2026/06/17/ASOS_20260617_0740_DavisTurner_0002.xml</t>
+  </si>
+  <si>
+    <t>49870000004093</t>
   </si>
   <si>
     <t>2026-07-16</t>
@@ -981,7 +981,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" s="2">
         <v>46192</v>
@@ -1044,13 +1044,13 @@
         <v>1.4</v>
       </c>
       <c r="Z2">
-        <v>200</v>
+        <v>6</v>
       </c>
       <c r="AA2">
         <v>0.072</v>
       </c>
       <c r="AB2">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="AC2" t="s">
         <v>45</v>
@@ -1545,16 +1545,16 @@
         <v>1</v>
       </c>
       <c r="AP2">
+        <v>3</v>
+      </c>
+      <c r="AQ2">
         <v>2</v>
-      </c>
-      <c r="AQ2">
-        <v>100</v>
       </c>
       <c r="AR2" s="3">
         <v>1.4</v>
       </c>
       <c r="AS2" s="3">
-        <v>200</v>
+        <v>6</v>
       </c>
       <c r="AT2" s="3">
         <v>0.072</v>
@@ -1949,7 +1949,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -2035,6 +2035,66 @@
         <v>39</v>
       </c>
     </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
removing stages wise ack of pipeline,manual feed
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="145">
   <si>
     <t>PO_Number</t>
   </si>
@@ -131,13 +131,10 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>500034236928</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>CY</t>
+    <t>CFS</t>
   </si>
   <si>
     <t>Road</t>
@@ -218,13 +215,16 @@
     <t>quantity</t>
   </si>
   <si>
-    <t>ASOS_20260617_0740_DavisTurner_0002.xml</t>
-  </si>
-  <si>
-    <t>ASNInDavisTurner/2026/06/17/ASOS_20260617_0740_DavisTurner_0002.xml</t>
-  </si>
-  <si>
-    <t>49870000004093</t>
+    <t>ASOS_20260617_0752_DavisTurner_0094.xml</t>
+  </si>
+  <si>
+    <t>ASNInDavisTurner/2026/06/17/ASOS_20260617_0752_DavisTurner_0094.xml</t>
+  </si>
+  <si>
+    <t>49870000004094</t>
+  </si>
+  <si>
+    <t>500034236929</t>
   </si>
   <si>
     <t>2026-07-16</t>
@@ -968,11 +968,11 @@
       </c>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>38</v>
+      <c r="A2">
+        <v>500034236929</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2">
         <v>148609059</v>
@@ -981,7 +981,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" s="2">
         <v>46192</v>
@@ -990,43 +990,43 @@
         <v>46193</v>
       </c>
       <c r="H2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s">
         <v>40</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>41</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>42</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T2" t="s">
         <v>43</v>
-      </c>
-      <c r="L2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N2" t="s">
-        <v>39</v>
-      </c>
-      <c r="O2" t="s">
-        <v>39</v>
-      </c>
-      <c r="P2" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>39</v>
-      </c>
-      <c r="R2" t="s">
-        <v>39</v>
-      </c>
-      <c r="S2" t="s">
-        <v>39</v>
-      </c>
-      <c r="T2" t="s">
-        <v>44</v>
       </c>
       <c r="U2">
         <v>60</v>
@@ -1044,43 +1044,43 @@
         <v>1.4</v>
       </c>
       <c r="Z2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="AA2">
         <v>0.072</v>
       </c>
       <c r="AB2">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="AC2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD2" t="s">
         <v>45</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AF2" t="s">
         <v>46</v>
       </c>
-      <c r="AE2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>47</v>
-      </c>
       <c r="AG2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AH2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AI2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AJ2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AK2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AL2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1099,78 +1099,78 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>68</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>69</v>
       </c>
-      <c r="D2" t="s">
-        <v>38</v>
-      </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
@@ -1422,16 +1422,16 @@
     </row>
     <row r="2" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
         <v>108</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
         <v>71</v>
@@ -1440,28 +1440,28 @@
         <v>72</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O2" t="s">
         <v>82</v>
@@ -1476,16 +1476,16 @@
         <v>111</v>
       </c>
       <c r="S2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="T2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="U2" t="s">
         <v>112</v>
       </c>
       <c r="V2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="W2" t="s">
         <v>113</v>
@@ -1497,7 +1497,7 @@
         <v>115</v>
       </c>
       <c r="Z2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA2" t="s">
         <v>73</v>
@@ -1527,7 +1527,7 @@
         <v>78</v>
       </c>
       <c r="AJ2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AK2" s="3">
         <v>60</v>
@@ -1545,34 +1545,34 @@
         <v>1</v>
       </c>
       <c r="AP2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AQ2">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="AR2" s="3">
         <v>1.4</v>
       </c>
       <c r="AS2" s="3">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="AT2" s="3">
         <v>0.072</v>
       </c>
       <c r="AU2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AV2" t="s">
         <v>45</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AW2" t="s">
         <v>46</v>
       </c>
-      <c r="AW2" t="s">
-        <v>47</v>
-      </c>
       <c r="AX2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AY2" t="s">
         <v>40</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>41</v>
       </c>
       <c r="AZ2" s="2">
         <v>46192</v>
@@ -1587,7 +1587,7 @@
         <v>116</v>
       </c>
       <c r="BD2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="BE2">
         <v>0</v>
@@ -1596,13 +1596,13 @@
         <v>0</v>
       </c>
       <c r="BG2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="BH2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="BI2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="BJ2" t="s">
         <v>74</v>
@@ -1644,7 +1644,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2">
         <v>1.4</v>
@@ -1949,7 +1949,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -1977,122 +1977,142 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
streamlining pipeline result,vb cancellation with PO input
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="145">
   <si>
     <t>PO_Number</t>
   </si>
@@ -1949,7 +1949,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -2115,6 +2115,106 @@
         <v>38</v>
       </c>
     </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Grouping upload & vb creation together and keeping cancellation separately,ref guide updates
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="145">
   <si>
     <t>PO_Number</t>
   </si>
@@ -1949,7 +1949,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -2215,6 +2215,26 @@
         <v>38</v>
       </c>
     </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
re-submission with latest vbref,clubbing cancel & re-submit
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="145">
   <si>
     <t>PO_Number</t>
   </si>
@@ -3114,7 +3114,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -5220,6 +5220,86 @@
         <v>39</v>
       </c>
     </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>39</v>
+      </c>
+      <c r="B106" t="s">
+        <v>39</v>
+      </c>
+      <c r="C106" t="s">
+        <v>39</v>
+      </c>
+      <c r="D106" t="s">
+        <v>39</v>
+      </c>
+      <c r="E106" t="s">
+        <v>39</v>
+      </c>
+      <c r="F106" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>39</v>
+      </c>
+      <c r="B107" t="s">
+        <v>39</v>
+      </c>
+      <c r="C107" t="s">
+        <v>39</v>
+      </c>
+      <c r="D107" t="s">
+        <v>39</v>
+      </c>
+      <c r="E107" t="s">
+        <v>39</v>
+      </c>
+      <c r="F107" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>39</v>
+      </c>
+      <c r="B108" t="s">
+        <v>39</v>
+      </c>
+      <c r="C108" t="s">
+        <v>39</v>
+      </c>
+      <c r="D108" t="s">
+        <v>39</v>
+      </c>
+      <c r="E108" t="s">
+        <v>39</v>
+      </c>
+      <c r="F108" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>39</v>
+      </c>
+      <c r="B109" t="s">
+        <v>39</v>
+      </c>
+      <c r="C109" t="s">
+        <v>39</v>
+      </c>
+      <c r="D109" t="s">
+        <v>39</v>
+      </c>
+      <c r="E109" t="s">
+        <v>39</v>
+      </c>
+      <c r="F109" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Manual upload test,auto upload wordings updated
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="92">
   <si>
     <t>PO_Number</t>
   </si>
@@ -140,304 +140,145 @@
     <t>CFS</t>
   </si>
   <si>
+    <t>Hanging</t>
+  </si>
+  <si>
+    <t>Bulk Flat</t>
+  </si>
+  <si>
+    <t>Delivery</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>filename</t>
+  </si>
+  <si>
+    <t>blobPath</t>
+  </si>
+  <si>
+    <t>asnId</t>
+  </si>
+  <si>
+    <t>poId</t>
+  </si>
+  <si>
+    <t>fcId</t>
+  </si>
+  <si>
+    <t>shipDate</t>
+  </si>
+  <si>
+    <t>supplier</t>
+  </si>
+  <si>
+    <t>supplierCode</t>
+  </si>
+  <si>
+    <t>shippingPoint</t>
+  </si>
+  <si>
+    <t>shippingTerms</t>
+  </si>
+  <si>
+    <t>sku</t>
+  </si>
+  <si>
+    <t>ean</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>colour</t>
+  </si>
+  <si>
+    <t>style</t>
+  </si>
+  <si>
+    <t>packFormat</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>Weight_KG</t>
+  </si>
+  <si>
+    <t>Length_cm</t>
+  </si>
+  <si>
+    <t>Width_cm</t>
+  </si>
+  <si>
+    <t>Height_cm</t>
+  </si>
+  <si>
     <t>BDCM1</t>
   </si>
   <si>
-    <t>Bulk Flat</t>
-  </si>
-  <si>
-    <t>Delivery</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>filename</t>
-  </si>
-  <si>
-    <t>blobPath</t>
-  </si>
-  <si>
-    <t>asnId</t>
-  </si>
-  <si>
-    <t>poId</t>
-  </si>
-  <si>
-    <t>fcId</t>
-  </si>
-  <si>
-    <t>shipDate</t>
-  </si>
-  <si>
-    <t>supplier</t>
-  </si>
-  <si>
-    <t>supplierCode</t>
-  </si>
-  <si>
-    <t>shippingPoint</t>
-  </si>
-  <si>
-    <t>shippingTerms</t>
-  </si>
-  <si>
-    <t>sku</t>
-  </si>
-  <si>
-    <t>ean</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>size</t>
-  </si>
-  <si>
-    <t>colour</t>
-  </si>
-  <si>
-    <t>style</t>
-  </si>
-  <si>
-    <t>packFormat</t>
-  </si>
-  <si>
-    <t>country</t>
-  </si>
-  <si>
-    <t>quantity</t>
-  </si>
-  <si>
-    <t>DATABRICKS_shipments.json</t>
-  </si>
-  <si>
-    <t>53470000055807</t>
-  </si>
-  <si>
-    <t>2026-06-25</t>
-  </si>
-  <si>
-    <t>Euro-Rose Group Limited (FCA)</t>
-  </si>
-  <si>
-    <t>2003175002</t>
-  </si>
-  <si>
-    <t>TRLEI</t>
-  </si>
-  <si>
-    <t>FCA</t>
-  </si>
-  <si>
-    <t>158726321</t>
-  </si>
-  <si>
-    <t>158726317</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>GB</t>
-  </si>
-  <si>
-    <t>158726324</t>
-  </si>
-  <si>
-    <t>158726327</t>
-  </si>
-  <si>
-    <t>158726330</t>
+    <t>BDCM3</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>Cartons</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>B4</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>Hanging Non-Standard</t>
+  </si>
+  <si>
+    <t>Non-Standard</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
   </si>
   <si>
     <t>Booking_Ref</t>
-  </si>
-  <si>
-    <t>Booking_Group</t>
-  </si>
-  <si>
-    <t>Supplier_Name</t>
-  </si>
-  <si>
-    <t>Supplier_ID</t>
-  </si>
-  <si>
-    <t>Supplier_Street1</t>
-  </si>
-  <si>
-    <t>Supplier_City</t>
-  </si>
-  <si>
-    <t>Supplier_PostalCd</t>
-  </si>
-  <si>
-    <t>Supplier_CountryCd</t>
-  </si>
-  <si>
-    <t>Factory_Street3</t>
-  </si>
-  <si>
-    <t>Country_Of_Origin</t>
-  </si>
-  <si>
-    <t>FC_ID</t>
-  </si>
-  <si>
-    <t>FC_Name</t>
-  </si>
-  <si>
-    <t>FC_Street1</t>
-  </si>
-  <si>
-    <t>FC_Street2</t>
-  </si>
-  <si>
-    <t>FC_Street3</t>
-  </si>
-  <si>
-    <t>FC_City</t>
-  </si>
-  <si>
-    <t>FC_StateProvinceCd</t>
-  </si>
-  <si>
-    <t>FC_PostalCd</t>
-  </si>
-  <si>
-    <t>FC_CountryCd</t>
-  </si>
-  <si>
-    <t>Carrier_ID</t>
-  </si>
-  <si>
-    <t>Carrier_Name</t>
-  </si>
-  <si>
-    <t>Loading_Port_LOCODE</t>
-  </si>
-  <si>
-    <t>POFC_ID</t>
-  </si>
-  <si>
-    <t>F1_ID</t>
-  </si>
-  <si>
-    <t>Product_Style</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Ship_Date</t>
-  </si>
-  <si>
-    <t>Incoterms</t>
-  </si>
-  <si>
-    <t>Transport_Mode_Code</t>
-  </si>
-  <si>
-    <t>Single Booking</t>
-  </si>
-  <si>
-    <t>F100774</t>
-  </si>
-  <si>
-    <t>Euro Rose Knitwear Limited</t>
-  </si>
-  <si>
-    <t>FC04</t>
-  </si>
-  <si>
-    <t>FC04 Berlin</t>
-  </si>
-  <si>
-    <t>An der Anhalter Bahn 6</t>
-  </si>
-  <si>
-    <t>Berlin</t>
-  </si>
-  <si>
-    <t>DE</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>2026-07-06</t>
-  </si>
-  <si>
-    <t>Weight_KG</t>
-  </si>
-  <si>
-    <t>Length_cm</t>
-  </si>
-  <si>
-    <t>Width_cm</t>
-  </si>
-  <si>
-    <t>Height_cm</t>
-  </si>
-  <si>
-    <t>BDCM3</t>
-  </si>
-  <si>
-    <t>C5</t>
-  </si>
-  <si>
-    <t>Cartons</t>
-  </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>A3</t>
-  </si>
-  <si>
-    <t>A4</t>
-  </si>
-  <si>
-    <t>B1</t>
-  </si>
-  <si>
-    <t>B2</t>
-  </si>
-  <si>
-    <t>B3</t>
-  </si>
-  <si>
-    <t>B4</t>
-  </si>
-  <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>C3</t>
-  </si>
-  <si>
-    <t>C4</t>
-  </si>
-  <si>
-    <t>Hanging</t>
-  </si>
-  <si>
-    <t>Hanging Non-Standard</t>
-  </si>
-  <si>
-    <t>Non-Standard</t>
-  </si>
-  <si>
-    <t>Timestamp</t>
   </si>
   <si>
     <t>PO_Numbers</t>
@@ -469,7 +310,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -479,11 +320,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -499,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -509,7 +345,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,7 +684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AL5"/>
+  <dimension ref="A1:AL2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
@@ -979,20 +814,20 @@
       <c r="B2" t="s">
         <v>39</v>
       </c>
-      <c r="C2">
-        <v>158726321</v>
+      <c r="C2" t="s">
+        <v>39</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>1009</v>
       </c>
       <c r="E2">
-        <v>0.29</v>
+        <v>3.8</v>
       </c>
       <c r="F2" s="4">
-        <v>46200</v>
+        <v>46230</v>
       </c>
       <c r="G2" s="4">
-        <v>46201</v>
+        <v>46231</v>
       </c>
       <c r="H2" t="s">
         <v>40</v>
@@ -1034,28 +869,28 @@
         <v>41</v>
       </c>
       <c r="U2">
+        <v>213</v>
+      </c>
+      <c r="V2">
+        <v>94</v>
+      </c>
+      <c r="W2">
         <v>60</v>
       </c>
-      <c r="V2">
-        <v>30</v>
-      </c>
-      <c r="W2">
-        <v>40</v>
-      </c>
       <c r="X2">
-        <v>1.4</v>
-      </c>
-      <c r="Y2">
-        <v>1.4</v>
-      </c>
-      <c r="Z2">
-        <v>2.61</v>
-      </c>
-      <c r="AA2">
-        <v>0.072</v>
-      </c>
-      <c r="AB2">
-        <v>9</v>
+        <v>0.7</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>39</v>
       </c>
       <c r="AC2" t="s">
         <v>42</v>
@@ -1085,354 +920,6 @@
         <v>39</v>
       </c>
       <c r="AL2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3">
-        <v>158726324</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>0.29</v>
-      </c>
-      <c r="F3" s="4">
-        <v>46200</v>
-      </c>
-      <c r="G3" s="4">
-        <v>46201</v>
-      </c>
-      <c r="H3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>39</v>
-      </c>
-      <c r="N3" t="s">
-        <v>39</v>
-      </c>
-      <c r="O3" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>39</v>
-      </c>
-      <c r="R3" t="s">
-        <v>39</v>
-      </c>
-      <c r="S3" t="s">
-        <v>39</v>
-      </c>
-      <c r="T3" t="s">
-        <v>41</v>
-      </c>
-      <c r="U3">
-        <v>60</v>
-      </c>
-      <c r="V3">
-        <v>30</v>
-      </c>
-      <c r="W3">
-        <v>40</v>
-      </c>
-      <c r="X3">
-        <v>1.4</v>
-      </c>
-      <c r="Y3">
-        <v>1.4</v>
-      </c>
-      <c r="Z3">
-        <v>8.41</v>
-      </c>
-      <c r="AA3">
-        <v>0.072</v>
-      </c>
-      <c r="AB3">
-        <v>29</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>44</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4">
-        <v>158726327</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>0.29</v>
-      </c>
-      <c r="F4" s="4">
-        <v>46200</v>
-      </c>
-      <c r="G4" s="4">
-        <v>46201</v>
-      </c>
-      <c r="H4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" t="s">
-        <v>39</v>
-      </c>
-      <c r="L4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M4" t="s">
-        <v>39</v>
-      </c>
-      <c r="N4" t="s">
-        <v>39</v>
-      </c>
-      <c r="O4" t="s">
-        <v>39</v>
-      </c>
-      <c r="P4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>39</v>
-      </c>
-      <c r="R4" t="s">
-        <v>39</v>
-      </c>
-      <c r="S4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T4" t="s">
-        <v>41</v>
-      </c>
-      <c r="U4">
-        <v>60</v>
-      </c>
-      <c r="V4">
-        <v>30</v>
-      </c>
-      <c r="W4">
-        <v>40</v>
-      </c>
-      <c r="X4">
-        <v>1.4</v>
-      </c>
-      <c r="Y4">
-        <v>1.4</v>
-      </c>
-      <c r="Z4">
-        <v>4.64</v>
-      </c>
-      <c r="AA4">
-        <v>0.072</v>
-      </c>
-      <c r="AB4">
-        <v>16</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>43</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>44</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5">
-        <v>158726330</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>0.29</v>
-      </c>
-      <c r="F5" s="4">
-        <v>46200</v>
-      </c>
-      <c r="G5" s="4">
-        <v>46201</v>
-      </c>
-      <c r="H5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" t="s">
-        <v>39</v>
-      </c>
-      <c r="L5" t="s">
-        <v>39</v>
-      </c>
-      <c r="M5" t="s">
-        <v>39</v>
-      </c>
-      <c r="N5" t="s">
-        <v>39</v>
-      </c>
-      <c r="O5" t="s">
-        <v>39</v>
-      </c>
-      <c r="P5" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>39</v>
-      </c>
-      <c r="R5" t="s">
-        <v>39</v>
-      </c>
-      <c r="S5" t="s">
-        <v>39</v>
-      </c>
-      <c r="T5" t="s">
-        <v>41</v>
-      </c>
-      <c r="U5">
-        <v>60</v>
-      </c>
-      <c r="V5">
-        <v>30</v>
-      </c>
-      <c r="W5">
-        <v>40</v>
-      </c>
-      <c r="X5">
-        <v>1.4</v>
-      </c>
-      <c r="Y5">
-        <v>1.4</v>
-      </c>
-      <c r="Z5">
-        <v>1.7399999999999998</v>
-      </c>
-      <c r="AA5">
-        <v>0.072</v>
-      </c>
-      <c r="AB5">
-        <v>6</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>43</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>44</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL5" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1444,7 +931,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="19" width="22" customWidth="1"/>
@@ -1509,242 +996,6 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H2" t="s">
-        <v>68</v>
-      </c>
-      <c r="I2" t="s">
-        <v>69</v>
-      </c>
-      <c r="J2" t="s">
-        <v>70</v>
-      </c>
-      <c r="K2" t="s">
-        <v>71</v>
-      </c>
-      <c r="L2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N2" t="s">
-        <v>39</v>
-      </c>
-      <c r="O2" t="s">
-        <v>39</v>
-      </c>
-      <c r="P2" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>73</v>
-      </c>
-      <c r="R2" t="s">
-        <v>74</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" t="s">
-        <v>67</v>
-      </c>
-      <c r="H3" t="s">
-        <v>68</v>
-      </c>
-      <c r="I3" t="s">
-        <v>69</v>
-      </c>
-      <c r="J3" t="s">
-        <v>70</v>
-      </c>
-      <c r="K3" t="s">
-        <v>75</v>
-      </c>
-      <c r="L3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>39</v>
-      </c>
-      <c r="N3" t="s">
-        <v>39</v>
-      </c>
-      <c r="O3" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>73</v>
-      </c>
-      <c r="R3" t="s">
-        <v>74</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" t="s">
-        <v>67</v>
-      </c>
-      <c r="H4" t="s">
-        <v>68</v>
-      </c>
-      <c r="I4" t="s">
-        <v>69</v>
-      </c>
-      <c r="J4" t="s">
-        <v>70</v>
-      </c>
-      <c r="K4" t="s">
-        <v>76</v>
-      </c>
-      <c r="L4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M4" t="s">
-        <v>39</v>
-      </c>
-      <c r="N4" t="s">
-        <v>39</v>
-      </c>
-      <c r="O4" t="s">
-        <v>39</v>
-      </c>
-      <c r="P4" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>73</v>
-      </c>
-      <c r="R4" t="s">
-        <v>74</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" t="s">
-        <v>67</v>
-      </c>
-      <c r="H5" t="s">
-        <v>68</v>
-      </c>
-      <c r="I5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J5" t="s">
-        <v>70</v>
-      </c>
-      <c r="K5" t="s">
-        <v>77</v>
-      </c>
-      <c r="L5" t="s">
-        <v>39</v>
-      </c>
-      <c r="M5" t="s">
-        <v>39</v>
-      </c>
-      <c r="N5" t="s">
-        <v>39</v>
-      </c>
-      <c r="O5" t="s">
-        <v>39</v>
-      </c>
-      <c r="P5" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>73</v>
-      </c>
-      <c r="R5" t="s">
-        <v>74</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1753,1029 +1004,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BO5"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="22" style="1" customWidth="1"/>
-    <col min="4" max="67" width="22" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AB1" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="AG1" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="AH1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="AJ1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="AK1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AL1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="AM1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="AN1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AO1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="AP1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="AQ1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="AR1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="AS1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AT1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="AU1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="AV1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="AW1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="AX1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AY1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="AZ1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="BA1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="BB1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="BC1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="BD1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="BF1" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="BG1" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="BH1" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="BI1" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="BJ1" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="BK1" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="BL1" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="BM1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="BN1" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="BO1" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I2" t="s">
-        <v>39</v>
-      </c>
-      <c r="J2" t="s">
-        <v>39</v>
-      </c>
-      <c r="K2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L2" t="s">
-        <v>109</v>
-      </c>
-      <c r="M2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N2" t="s">
-        <v>39</v>
-      </c>
-      <c r="O2" t="s">
-        <v>39</v>
-      </c>
-      <c r="P2" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>39</v>
-      </c>
-      <c r="R2" t="s">
-        <v>39</v>
-      </c>
-      <c r="S2" t="s">
-        <v>74</v>
-      </c>
-      <c r="T2" t="s">
-        <v>110</v>
-      </c>
-      <c r="U2" t="s">
-        <v>111</v>
-      </c>
-      <c r="V2" t="s">
-        <v>112</v>
-      </c>
-      <c r="W2" t="s">
-        <v>39</v>
-      </c>
-      <c r="X2" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>113</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>114</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>115</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>110</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>110</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>71</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AO2" s="5">
-        <v>60</v>
-      </c>
-      <c r="AP2" s="5">
-        <v>30</v>
-      </c>
-      <c r="AQ2" s="5">
-        <v>40</v>
-      </c>
-      <c r="AR2" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AS2">
-        <v>1</v>
-      </c>
-      <c r="AT2">
-        <v>0.29</v>
-      </c>
-      <c r="AU2">
-        <v>9</v>
-      </c>
-      <c r="AV2" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AW2" s="5">
-        <v>2.61</v>
-      </c>
-      <c r="AX2" s="5">
-        <v>0.072</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>42</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>43</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>44</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>40</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>116</v>
-      </c>
-      <c r="BD2" s="4">
-        <v>46200</v>
-      </c>
-      <c r="BE2" s="4">
-        <v>46201</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>66</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>117</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>39</v>
-      </c>
-      <c r="BI2">
-        <v>0</v>
-      </c>
-      <c r="BJ2">
-        <v>0</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>39</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>39</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>39</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>70</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="3" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E3" t="s">
-        <v>67</v>
-      </c>
-      <c r="F3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" t="s">
-        <v>108</v>
-      </c>
-      <c r="L3" t="s">
-        <v>109</v>
-      </c>
-      <c r="M3" t="s">
-        <v>39</v>
-      </c>
-      <c r="N3" t="s">
-        <v>39</v>
-      </c>
-      <c r="O3" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>39</v>
-      </c>
-      <c r="R3" t="s">
-        <v>39</v>
-      </c>
-      <c r="S3" t="s">
-        <v>74</v>
-      </c>
-      <c r="T3" t="s">
-        <v>110</v>
-      </c>
-      <c r="U3" t="s">
-        <v>111</v>
-      </c>
-      <c r="V3" t="s">
-        <v>112</v>
-      </c>
-      <c r="W3" t="s">
-        <v>39</v>
-      </c>
-      <c r="X3" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>113</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>114</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>115</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>69</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>110</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>110</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>75</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AO3" s="5">
-        <v>60</v>
-      </c>
-      <c r="AP3" s="5">
-        <v>30</v>
-      </c>
-      <c r="AQ3" s="5">
-        <v>40</v>
-      </c>
-      <c r="AR3" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AS3">
-        <v>1</v>
-      </c>
-      <c r="AT3">
-        <v>0.29</v>
-      </c>
-      <c r="AU3">
-        <v>29</v>
-      </c>
-      <c r="AV3" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AW3" s="5">
-        <v>8.41</v>
-      </c>
-      <c r="AX3" s="5">
-        <v>0.072</v>
-      </c>
-      <c r="AY3" t="s">
-        <v>42</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>43</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>44</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>40</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>116</v>
-      </c>
-      <c r="BD3" s="4">
-        <v>46200</v>
-      </c>
-      <c r="BE3" s="4">
-        <v>46201</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>66</v>
-      </c>
-      <c r="BG3" t="s">
-        <v>117</v>
-      </c>
-      <c r="BH3" t="s">
-        <v>39</v>
-      </c>
-      <c r="BI3">
-        <v>0</v>
-      </c>
-      <c r="BJ3">
-        <v>0</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>39</v>
-      </c>
-      <c r="BL3" t="s">
-        <v>39</v>
-      </c>
-      <c r="BM3" t="s">
-        <v>39</v>
-      </c>
-      <c r="BN3" t="s">
-        <v>70</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="4" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" t="s">
-        <v>108</v>
-      </c>
-      <c r="L4" t="s">
-        <v>109</v>
-      </c>
-      <c r="M4" t="s">
-        <v>39</v>
-      </c>
-      <c r="N4" t="s">
-        <v>39</v>
-      </c>
-      <c r="O4" t="s">
-        <v>39</v>
-      </c>
-      <c r="P4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>39</v>
-      </c>
-      <c r="R4" t="s">
-        <v>39</v>
-      </c>
-      <c r="S4" t="s">
-        <v>74</v>
-      </c>
-      <c r="T4" t="s">
-        <v>110</v>
-      </c>
-      <c r="U4" t="s">
-        <v>111</v>
-      </c>
-      <c r="V4" t="s">
-        <v>112</v>
-      </c>
-      <c r="W4" t="s">
-        <v>39</v>
-      </c>
-      <c r="X4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>113</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>114</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>115</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>69</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>76</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>41</v>
-      </c>
-      <c r="AO4" s="5">
-        <v>60</v>
-      </c>
-      <c r="AP4" s="5">
-        <v>30</v>
-      </c>
-      <c r="AQ4" s="5">
-        <v>40</v>
-      </c>
-      <c r="AR4" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AS4">
-        <v>1</v>
-      </c>
-      <c r="AT4">
-        <v>0.29</v>
-      </c>
-      <c r="AU4">
-        <v>16</v>
-      </c>
-      <c r="AV4" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AW4" s="5">
-        <v>4.64</v>
-      </c>
-      <c r="AX4" s="5">
-        <v>0.072</v>
-      </c>
-      <c r="AY4" t="s">
-        <v>42</v>
-      </c>
-      <c r="AZ4" t="s">
-        <v>43</v>
-      </c>
-      <c r="BA4" t="s">
-        <v>44</v>
-      </c>
-      <c r="BB4" t="s">
-        <v>40</v>
-      </c>
-      <c r="BC4" t="s">
-        <v>116</v>
-      </c>
-      <c r="BD4" s="4">
-        <v>46200</v>
-      </c>
-      <c r="BE4" s="4">
-        <v>46201</v>
-      </c>
-      <c r="BF4" t="s">
-        <v>66</v>
-      </c>
-      <c r="BG4" t="s">
-        <v>117</v>
-      </c>
-      <c r="BH4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BI4">
-        <v>0</v>
-      </c>
-      <c r="BJ4">
-        <v>0</v>
-      </c>
-      <c r="BK4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BL4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BM4" t="s">
-        <v>39</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>70</v>
-      </c>
-      <c r="BO4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="5" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E5" t="s">
-        <v>67</v>
-      </c>
-      <c r="F5" t="s">
-        <v>68</v>
-      </c>
-      <c r="G5" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" t="s">
-        <v>108</v>
-      </c>
-      <c r="L5" t="s">
-        <v>109</v>
-      </c>
-      <c r="M5" t="s">
-        <v>39</v>
-      </c>
-      <c r="N5" t="s">
-        <v>39</v>
-      </c>
-      <c r="O5" t="s">
-        <v>39</v>
-      </c>
-      <c r="P5" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>39</v>
-      </c>
-      <c r="R5" t="s">
-        <v>39</v>
-      </c>
-      <c r="S5" t="s">
-        <v>74</v>
-      </c>
-      <c r="T5" t="s">
-        <v>110</v>
-      </c>
-      <c r="U5" t="s">
-        <v>111</v>
-      </c>
-      <c r="V5" t="s">
-        <v>112</v>
-      </c>
-      <c r="W5" t="s">
-        <v>39</v>
-      </c>
-      <c r="X5" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>113</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>114</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>115</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>69</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>110</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>110</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>77</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>41</v>
-      </c>
-      <c r="AO5" s="5">
-        <v>60</v>
-      </c>
-      <c r="AP5" s="5">
-        <v>30</v>
-      </c>
-      <c r="AQ5" s="5">
-        <v>40</v>
-      </c>
-      <c r="AR5" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AS5">
-        <v>1</v>
-      </c>
-      <c r="AT5">
-        <v>0.29</v>
-      </c>
-      <c r="AU5">
-        <v>6</v>
-      </c>
-      <c r="AV5" s="5">
-        <v>1.4</v>
-      </c>
-      <c r="AW5" s="5">
-        <v>1.74</v>
-      </c>
-      <c r="AX5" s="5">
-        <v>0.072</v>
-      </c>
-      <c r="AY5" t="s">
-        <v>42</v>
-      </c>
-      <c r="AZ5" t="s">
-        <v>43</v>
-      </c>
-      <c r="BA5" t="s">
-        <v>44</v>
-      </c>
-      <c r="BB5" t="s">
-        <v>40</v>
-      </c>
-      <c r="BC5" t="s">
-        <v>116</v>
-      </c>
-      <c r="BD5" s="4">
-        <v>46200</v>
-      </c>
-      <c r="BE5" s="4">
-        <v>46201</v>
-      </c>
-      <c r="BF5" t="s">
-        <v>66</v>
-      </c>
-      <c r="BG5" t="s">
-        <v>117</v>
-      </c>
-      <c r="BH5" t="s">
-        <v>39</v>
-      </c>
-      <c r="BI5">
-        <v>0</v>
-      </c>
-      <c r="BJ5">
-        <v>0</v>
-      </c>
-      <c r="BK5" t="s">
-        <v>39</v>
-      </c>
-      <c r="BL5" t="s">
-        <v>39</v>
-      </c>
-      <c r="BM5" t="s">
-        <v>39</v>
-      </c>
-      <c r="BN5" t="s">
-        <v>70</v>
-      </c>
-      <c r="BO5" t="s">
-        <v>116</v>
-      </c>
-    </row>
+    <row r="1" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2795,21 +1027,21 @@
         <v>19</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>118</v>
+        <v>64</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>119</v>
+        <v>65</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>121</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="B2">
         <v>1.4</v>
@@ -2826,7 +1058,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>122</v>
+        <v>69</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -2843,7 +1075,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>70</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -2860,7 +1092,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>71</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -2877,7 +1109,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>72</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -2894,7 +1126,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>126</v>
+        <v>73</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -2911,7 +1143,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>74</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -2928,7 +1160,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -2945,7 +1177,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>129</v>
+        <v>76</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -2962,7 +1194,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>77</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -2979,7 +1211,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>131</v>
+        <v>78</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -2996,7 +1228,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -3013,7 +1245,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -3030,7 +1262,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -3047,7 +1279,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>135</v>
+        <v>82</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -3064,7 +1296,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>136</v>
+        <v>83</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -3081,7 +1313,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>137</v>
+        <v>41</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -3098,12 +1330,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>138</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>139</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -3114,7 +1346,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -3122,22 +1354,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>140</v>
+        <v>86</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>141</v>
+        <v>88</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>142</v>
+        <v>89</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>143</v>
+        <v>90</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>144</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -5297,6 +3529,26 @@
         <v>39</v>
       </c>
       <c r="F109" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>39</v>
+      </c>
+      <c r="B110" t="s">
+        <v>39</v>
+      </c>
+      <c r="C110" t="s">
+        <v>39</v>
+      </c>
+      <c r="D110" t="s">
+        <v>39</v>
+      </c>
+      <c r="E110" t="s">
+        <v>39</v>
+      </c>
+      <c r="F110" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Extra SKU booked =0 notification is removed,valid booking qty
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1448" uniqueCount="157">
   <si>
     <t>PO_Number</t>
   </si>
@@ -131,7 +131,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>500037528092</t>
+    <t>500037691135</t>
   </si>
   <si>
     <t/>
@@ -140,135 +140,333 @@
     <t>CFS</t>
   </si>
   <si>
+    <t>BDCM1</t>
+  </si>
+  <si>
+    <t>Bulk Flat</t>
+  </si>
+  <si>
+    <t>Delivery</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>500037691136</t>
+  </si>
+  <si>
+    <t>filename</t>
+  </si>
+  <si>
+    <t>blobPath</t>
+  </si>
+  <si>
+    <t>asnId</t>
+  </si>
+  <si>
+    <t>poId</t>
+  </si>
+  <si>
+    <t>fcId</t>
+  </si>
+  <si>
+    <t>shipDate</t>
+  </si>
+  <si>
+    <t>supplier</t>
+  </si>
+  <si>
+    <t>supplierCode</t>
+  </si>
+  <si>
+    <t>shippingPoint</t>
+  </si>
+  <si>
+    <t>shippingTerms</t>
+  </si>
+  <si>
+    <t>sku</t>
+  </si>
+  <si>
+    <t>ean</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>colour</t>
+  </si>
+  <si>
+    <t>style</t>
+  </si>
+  <si>
+    <t>packFormat</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>DATABRICKS_shipments.json</t>
+  </si>
+  <si>
+    <t>49870000067054</t>
+  </si>
+  <si>
+    <t>2026-07-17</t>
+  </si>
+  <si>
+    <t>Cherryfield Trading Ltd (USD)</t>
+  </si>
+  <si>
+    <t>1100001085</t>
+  </si>
+  <si>
+    <t>TRIST</t>
+  </si>
+  <si>
+    <t>FOB</t>
+  </si>
+  <si>
+    <t>159194209</t>
+  </si>
+  <si>
+    <t>159194194</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>159194225</t>
+  </si>
+  <si>
+    <t>159194228</t>
+  </si>
+  <si>
+    <t>159194255</t>
+  </si>
+  <si>
+    <t>49870000067059</t>
+  </si>
+  <si>
+    <t>2026-07-15</t>
+  </si>
+  <si>
+    <t>Booking_Ref</t>
+  </si>
+  <si>
+    <t>Booking_Group</t>
+  </si>
+  <si>
+    <t>_missingFromSupplier</t>
+  </si>
+  <si>
+    <t>Supplier_Name</t>
+  </si>
+  <si>
+    <t>Supplier_ID</t>
+  </si>
+  <si>
+    <t>Supplier_Street1</t>
+  </si>
+  <si>
+    <t>Supplier_City</t>
+  </si>
+  <si>
+    <t>Supplier_PostalCd</t>
+  </si>
+  <si>
+    <t>Supplier_CountryCd</t>
+  </si>
+  <si>
+    <t>Factory_Street3</t>
+  </si>
+  <si>
+    <t>Country_Of_Origin</t>
+  </si>
+  <si>
+    <t>FC_ID</t>
+  </si>
+  <si>
+    <t>FC_Name</t>
+  </si>
+  <si>
+    <t>FC_Street1</t>
+  </si>
+  <si>
+    <t>FC_Street2</t>
+  </si>
+  <si>
+    <t>FC_Street3</t>
+  </si>
+  <si>
+    <t>FC_City</t>
+  </si>
+  <si>
+    <t>FC_StateProvinceCd</t>
+  </si>
+  <si>
+    <t>FC_PostalCd</t>
+  </si>
+  <si>
+    <t>FC_CountryCd</t>
+  </si>
+  <si>
+    <t>Carrier_ID</t>
+  </si>
+  <si>
+    <t>Carrier_Name</t>
+  </si>
+  <si>
+    <t>Loading_Port_LOCODE</t>
+  </si>
+  <si>
+    <t>POFC_ID</t>
+  </si>
+  <si>
+    <t>F1_ID</t>
+  </si>
+  <si>
+    <t>Product_Style</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>PO_Header_Cartons</t>
+  </si>
+  <si>
+    <t>PO_Header_UnitWeight</t>
+  </si>
+  <si>
+    <t>PO_Header_CartonType</t>
+  </si>
+  <si>
+    <t>Ship_Date</t>
+  </si>
+  <si>
+    <t>Incoterms</t>
+  </si>
+  <si>
+    <t>Transport_Mode_Code</t>
+  </si>
+  <si>
+    <t>Single Booking</t>
+  </si>
+  <si>
+    <t>FC04</t>
+  </si>
+  <si>
+    <t>FC04 Berlin</t>
+  </si>
+  <si>
+    <t>An der Anhalter Bahn 6</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>2026-07-18</t>
+  </si>
+  <si>
+    <t>FC01</t>
+  </si>
+  <si>
+    <t>ASOS Barnsley</t>
+  </si>
+  <si>
+    <t>Langthwaite Grange Industrial Estate</t>
+  </si>
+  <si>
+    <t>South Kirkby</t>
+  </si>
+  <si>
+    <t>WF9 3NR</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>2026-07-23</t>
+  </si>
+  <si>
+    <t>Weight_KG</t>
+  </si>
+  <si>
+    <t>Length_cm</t>
+  </si>
+  <si>
+    <t>Width_cm</t>
+  </si>
+  <si>
+    <t>Height_cm</t>
+  </si>
+  <si>
+    <t>BDCM3</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>Cartons</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>B4</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
     <t>Hanging</t>
   </si>
   <si>
-    <t>Bulk Flat</t>
-  </si>
-  <si>
-    <t>Delivery</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>filename</t>
-  </si>
-  <si>
-    <t>blobPath</t>
-  </si>
-  <si>
-    <t>asnId</t>
-  </si>
-  <si>
-    <t>poId</t>
-  </si>
-  <si>
-    <t>fcId</t>
-  </si>
-  <si>
-    <t>shipDate</t>
-  </si>
-  <si>
-    <t>supplier</t>
-  </si>
-  <si>
-    <t>supplierCode</t>
-  </si>
-  <si>
-    <t>shippingPoint</t>
-  </si>
-  <si>
-    <t>shippingTerms</t>
-  </si>
-  <si>
-    <t>sku</t>
-  </si>
-  <si>
-    <t>ean</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>size</t>
-  </si>
-  <si>
-    <t>colour</t>
-  </si>
-  <si>
-    <t>style</t>
-  </si>
-  <si>
-    <t>packFormat</t>
-  </si>
-  <si>
-    <t>country</t>
-  </si>
-  <si>
-    <t>quantity</t>
-  </si>
-  <si>
-    <t>Weight_KG</t>
-  </si>
-  <si>
-    <t>Length_cm</t>
-  </si>
-  <si>
-    <t>Width_cm</t>
-  </si>
-  <si>
-    <t>Height_cm</t>
-  </si>
-  <si>
-    <t>BDCM1</t>
-  </si>
-  <si>
-    <t>BDCM3</t>
-  </si>
-  <si>
-    <t>C5</t>
-  </si>
-  <si>
-    <t>Cartons</t>
-  </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>A3</t>
-  </si>
-  <si>
-    <t>A4</t>
-  </si>
-  <si>
-    <t>B1</t>
-  </si>
-  <si>
-    <t>B2</t>
-  </si>
-  <si>
-    <t>B3</t>
-  </si>
-  <si>
-    <t>B4</t>
-  </si>
-  <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>C3</t>
-  </si>
-  <si>
-    <t>C4</t>
-  </si>
-  <si>
     <t>Hanging Non-Standard</t>
   </si>
   <si>
@@ -276,9 +474,6 @@
   </si>
   <si>
     <t>Timestamp</t>
-  </si>
-  <si>
-    <t>Booking_Ref</t>
   </si>
   <si>
     <t>PO_Numbers</t>
@@ -310,7 +505,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -320,6 +515,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -335,7 +540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -345,6 +550,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AL2"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
@@ -818,16 +1027,16 @@
         <v>39</v>
       </c>
       <c r="D2">
-        <v>1009</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>3.8</v>
+        <v>0.21</v>
       </c>
       <c r="F2" s="4">
-        <v>46230</v>
+        <v>46213</v>
       </c>
       <c r="G2" s="4">
-        <v>46231</v>
+        <v>46213</v>
       </c>
       <c r="H2" t="s">
         <v>40</v>
@@ -869,16 +1078,16 @@
         <v>41</v>
       </c>
       <c r="U2">
-        <v>213</v>
+        <v>60</v>
       </c>
       <c r="V2">
-        <v>94</v>
+        <v>30</v>
       </c>
       <c r="W2">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="X2">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="Y2" t="s">
         <v>39</v>
@@ -920,6 +1129,122 @@
         <v>39</v>
       </c>
       <c r="AL2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>0.21</v>
+      </c>
+      <c r="F3" s="4">
+        <v>46213</v>
+      </c>
+      <c r="G3" s="4">
+        <v>46213</v>
+      </c>
+      <c r="H3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>39</v>
+      </c>
+      <c r="R3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" t="s">
+        <v>39</v>
+      </c>
+      <c r="T3" t="s">
+        <v>41</v>
+      </c>
+      <c r="U3">
+        <v>60</v>
+      </c>
+      <c r="V3">
+        <v>30</v>
+      </c>
+      <c r="W3">
+        <v>40</v>
+      </c>
+      <c r="X3">
+        <v>1.4</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -931,7 +1256,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="19" width="22" customWidth="1"/>
@@ -939,61 +1264,533 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>63</v>
+      <c r="E2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J2" t="s">
+        <v>71</v>
+      </c>
+      <c r="K2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>74</v>
+      </c>
+      <c r="R2" t="s">
+        <v>75</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" t="s">
+        <v>70</v>
+      </c>
+      <c r="J3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>74</v>
+      </c>
+      <c r="R3" t="s">
+        <v>75</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J4" t="s">
+        <v>71</v>
+      </c>
+      <c r="K4" t="s">
+        <v>77</v>
+      </c>
+      <c r="L4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>74</v>
+      </c>
+      <c r="R4" t="s">
+        <v>75</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>67</v>
+      </c>
+      <c r="G5" t="s">
+        <v>68</v>
+      </c>
+      <c r="H5" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" t="s">
+        <v>70</v>
+      </c>
+      <c r="J5" t="s">
+        <v>71</v>
+      </c>
+      <c r="K5" t="s">
+        <v>78</v>
+      </c>
+      <c r="L5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P5" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>74</v>
+      </c>
+      <c r="R5" t="s">
+        <v>75</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" t="s">
+        <v>70</v>
+      </c>
+      <c r="J6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L6" t="s">
+        <v>39</v>
+      </c>
+      <c r="M6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" t="s">
+        <v>39</v>
+      </c>
+      <c r="O6" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>74</v>
+      </c>
+      <c r="R6" t="s">
+        <v>75</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" t="s">
+        <v>70</v>
+      </c>
+      <c r="J7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K7" t="s">
+        <v>76</v>
+      </c>
+      <c r="L7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M7" t="s">
+        <v>39</v>
+      </c>
+      <c r="N7" t="s">
+        <v>39</v>
+      </c>
+      <c r="O7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P7" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>74</v>
+      </c>
+      <c r="R7" t="s">
+        <v>75</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G8" t="s">
+        <v>68</v>
+      </c>
+      <c r="H8" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" t="s">
+        <v>70</v>
+      </c>
+      <c r="J8" t="s">
+        <v>71</v>
+      </c>
+      <c r="K8" t="s">
+        <v>77</v>
+      </c>
+      <c r="L8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M8" t="s">
+        <v>39</v>
+      </c>
+      <c r="N8" t="s">
+        <v>39</v>
+      </c>
+      <c r="O8" t="s">
+        <v>39</v>
+      </c>
+      <c r="P8" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>74</v>
+      </c>
+      <c r="R8" t="s">
+        <v>75</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" t="s">
+        <v>71</v>
+      </c>
+      <c r="K9" t="s">
+        <v>78</v>
+      </c>
+      <c r="L9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" t="s">
+        <v>39</v>
+      </c>
+      <c r="N9" t="s">
+        <v>39</v>
+      </c>
+      <c r="O9" t="s">
+        <v>39</v>
+      </c>
+      <c r="P9" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>74</v>
+      </c>
+      <c r="R9" t="s">
+        <v>75</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1004,10 +1801,1949 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:BS9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" style="1" customWidth="1"/>
+    <col min="4" max="71" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1" ht="20" customHeight="1" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AG1" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="AH1" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AI1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="AJ1" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AK1" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="AL1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="AM1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="AO1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AP1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="AR1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="AS1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="AT1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="AU1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="AV1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AW1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AX1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="AY1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="AZ1" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="BA1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="BB1" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="BC1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="BD1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="BE1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="BF1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="BG1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="BH1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="BI1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="BJ1" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="BK1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="BL1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="BM1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="BN1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="BO1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="BP1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="BQ1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="BR1" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="BS1" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z2" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="AA2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC2" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="AD2" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG2" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH2" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="AJ2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP2" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ2" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR2" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS2" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT2" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU2" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV2" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW2" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY2" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ2" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA2" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG2" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH2" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI2" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ2" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BK2" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="BL2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM2" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN2" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR2" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS2" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC3" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="AD3" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG3" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH3" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AJ3" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP3" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ3" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR3" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS3" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT3" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU3" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW3" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY3" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ3" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA3" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG3" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH3" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI3" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ3" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BK3" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="BL3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM3" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN3" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS3" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC4" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="AD4" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF4" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI4" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AJ4" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP4" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ4" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR4" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS4" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT4" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU4" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV4" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW4" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY4" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ4" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA4" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG4" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH4" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI4" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BK4" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="BL4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM4" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN4" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR4" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS4" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC5" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="AD5" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF5" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG5" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AH5" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI5" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ5" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP5" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ5" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR5" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS5" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT5" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU5" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV5" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW5" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX5" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY5" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ5" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA5" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG5" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH5" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI5" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ5" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BK5" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="BL5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM5" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN5" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR5" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS5" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC6" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD6" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG6" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AH6" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AI6" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="AJ6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP6" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ6" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR6" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS6" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT6" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU6" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV6" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW6" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX6" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY6" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ6" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA6" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC6" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE6" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH6" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI6" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ6" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="BK6" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="BL6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM6" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN6" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS6" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U7" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="AA7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC7" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD7" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF7" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG7" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AH7" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AI7" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AJ7" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP7" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ7" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR7" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS7" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT7" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU7" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV7" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW7" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX7" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY7" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ7" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA7" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG7" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH7" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI7" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ7" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="BK7" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="BL7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM7" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN7" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR7" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS7" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U8" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC8" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD8" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF8" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG8" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AH8" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AI8" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AJ8" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP8" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ8" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR8" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS8" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT8" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU8" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV8" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW8" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX8" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY8" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ8" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA8" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC8" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE8" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG8" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH8" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI8" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ8" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="BK8" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="BL8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM8" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN8" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR8" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS8" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:71" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T9" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="U9" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="V9" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="W9" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="AA9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB9" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC9" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD9" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF9" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG9" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AH9" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AI9" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ9" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AL9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP9" s="7">
+        <v>60</v>
+      </c>
+      <c r="AQ9" s="7">
+        <v>30</v>
+      </c>
+      <c r="AR9" s="7">
+        <v>40</v>
+      </c>
+      <c r="AS9" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AT9" s="5">
+        <v>1</v>
+      </c>
+      <c r="AU9" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="AV9" s="5">
+        <v>0</v>
+      </c>
+      <c r="AW9" s="7">
+        <v>1.4</v>
+      </c>
+      <c r="AX9" s="7">
+        <v>0</v>
+      </c>
+      <c r="AY9" s="7">
+        <v>0.072</v>
+      </c>
+      <c r="AZ9" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA9" s="5">
+        <v>0.21</v>
+      </c>
+      <c r="BB9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC9" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BD9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="BE9" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG9" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH9" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BI9" s="8">
+        <v>46213</v>
+      </c>
+      <c r="BJ9" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="BK9" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="BL9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BM9" s="5">
+        <v>0</v>
+      </c>
+      <c r="BN9" s="5">
+        <v>0</v>
+      </c>
+      <c r="BO9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BP9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="BR9" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="BS9" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1027,21 +3763,21 @@
         <v>19</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>65</v>
+        <v>131</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>66</v>
+        <v>132</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>67</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="B2">
         <v>1.4</v>
@@ -1058,7 +3794,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>134</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1075,7 +3811,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>135</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1092,7 +3828,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>136</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1109,7 +3845,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>137</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1126,7 +3862,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>138</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1143,7 +3879,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>139</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1160,7 +3896,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>75</v>
+        <v>140</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1177,7 +3913,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>141</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1194,7 +3930,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>142</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1211,7 +3947,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>143</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1228,7 +3964,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>79</v>
+        <v>144</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1245,7 +3981,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>145</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1262,7 +3998,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>146</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1279,7 +4015,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>147</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1296,7 +4032,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>83</v>
+        <v>148</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1313,7 +4049,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>149</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -1330,12 +4066,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -1354,22 +4090,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>86</v>
+        <v>152</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>88</v>
+        <v>153</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>89</v>
+        <v>154</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>91</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ref guide updated,result SKU count fixed,BKDQty lookup, SKU description,Measure N, G fix,VB code
</commit_message>
<xml_diff>
--- a/bible/SupplierBible_working.xlsx
+++ b/bible/SupplierBible_working.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1448" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1472" uniqueCount="158">
   <si>
     <t>PO_Number</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>159194209</t>
+  </si>
+  <si>
+    <t>ASOS DESIGN relaxed sweatshirt with collegiate front print in blue</t>
   </si>
   <si>
     <t>159194194</t>
@@ -1030,7 +1033,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="F2" s="4">
         <v>46213</v>
@@ -1146,7 +1149,7 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="F3" s="4">
         <v>46213</v>
@@ -1359,7 +1362,7 @@
         <v>39</v>
       </c>
       <c r="M2" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="N2" t="s">
         <v>39</v>
@@ -1368,16 +1371,16 @@
         <v>39</v>
       </c>
       <c r="P2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S2">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -1412,31 +1415,31 @@
         <v>71</v>
       </c>
       <c r="K3" t="s">
+        <v>77</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>75</v>
+      </c>
+      <c r="R3" t="s">
         <v>76</v>
       </c>
-      <c r="L3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>39</v>
-      </c>
-      <c r="N3" t="s">
-        <v>39</v>
-      </c>
-      <c r="O3" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>74</v>
-      </c>
-      <c r="R3" t="s">
-        <v>75</v>
-      </c>
       <c r="S3">
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -1471,13 +1474,13 @@
         <v>71</v>
       </c>
       <c r="K4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L4" t="s">
         <v>39</v>
       </c>
       <c r="M4" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="N4" t="s">
         <v>39</v>
@@ -1486,16 +1489,16 @@
         <v>39</v>
       </c>
       <c r="P4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1530,13 +1533,13 @@
         <v>71</v>
       </c>
       <c r="K5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="L5" t="s">
         <v>39</v>
       </c>
       <c r="M5" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="N5" t="s">
         <v>39</v>
@@ -1545,16 +1548,16 @@
         <v>39</v>
       </c>
       <c r="P5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -1565,7 +1568,7 @@
         <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D6" t="s">
         <v>38</v>
@@ -1574,7 +1577,7 @@
         <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G6" t="s">
         <v>68</v>
@@ -1595,7 +1598,7 @@
         <v>39</v>
       </c>
       <c r="M6" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="N6" t="s">
         <v>39</v>
@@ -1604,16 +1607,16 @@
         <v>39</v>
       </c>
       <c r="P6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -1624,7 +1627,7 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
         <v>38</v>
@@ -1633,7 +1636,7 @@
         <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G7" t="s">
         <v>68</v>
@@ -1648,31 +1651,31 @@
         <v>71</v>
       </c>
       <c r="K7" t="s">
+        <v>77</v>
+      </c>
+      <c r="L7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M7" t="s">
+        <v>73</v>
+      </c>
+      <c r="N7" t="s">
+        <v>39</v>
+      </c>
+      <c r="O7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P7" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>75</v>
+      </c>
+      <c r="R7" t="s">
         <v>76</v>
       </c>
-      <c r="L7" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" t="s">
-        <v>39</v>
-      </c>
-      <c r="N7" t="s">
-        <v>39</v>
-      </c>
-      <c r="O7" t="s">
-        <v>39</v>
-      </c>
-      <c r="P7" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>74</v>
-      </c>
-      <c r="R7" t="s">
-        <v>75</v>
-      </c>
       <c r="S7">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -1683,7 +1686,7 @@
         <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
         <v>38</v>
@@ -1692,7 +1695,7 @@
         <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G8" t="s">
         <v>68</v>
@@ -1707,13 +1710,13 @@
         <v>71</v>
       </c>
       <c r="K8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L8" t="s">
         <v>39</v>
       </c>
       <c r="M8" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="N8" t="s">
         <v>39</v>
@@ -1722,16 +1725,16 @@
         <v>39</v>
       </c>
       <c r="P8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S8">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -1742,7 +1745,7 @@
         <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
         <v>38</v>
@@ -1751,7 +1754,7 @@
         <v>39</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
         <v>68</v>
@@ -1766,13 +1769,13 @@
         <v>71</v>
       </c>
       <c r="K9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="L9" t="s">
         <v>39</v>
       </c>
       <c r="M9" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="N9" t="s">
         <v>39</v>
@@ -1781,16 +1784,16 @@
         <v>39</v>
       </c>
       <c r="P9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1811,10 +1814,10 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:71" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -1823,25 +1826,25 @@
         <v>1</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>9</v>
@@ -1856,7 +1859,7 @@
         <v>12</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q1" s="3" t="s">
         <v>13</v>
@@ -1868,58 +1871,58 @@
         <v>15</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AB1" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AD1" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AE1" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AF1" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AI1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AL1" s="3" t="s">
         <v>16</v>
@@ -1964,13 +1967,13 @@
         <v>26</v>
       </c>
       <c r="AZ1" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BA1" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BB1" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BC1" s="3" t="s">
         <v>28</v>
@@ -1994,7 +1997,7 @@
         <v>6</v>
       </c>
       <c r="BJ1" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BK1" s="3" t="s">
         <v>32</v>
@@ -2018,10 +2021,10 @@
         <v>30</v>
       </c>
       <c r="BR1" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="BS1" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:71" x14ac:dyDescent="0.25">
@@ -2029,7 +2032,7 @@
         <v>39</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>45</v>
@@ -2083,16 +2086,16 @@
         <v>39</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X2" s="5" t="s">
         <v>39</v>
@@ -2101,7 +2104,7 @@
         <v>39</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA2" s="5" t="s">
         <v>39</v>
@@ -2110,10 +2113,10 @@
         <v>39</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AD2" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE2" s="5" t="s">
         <v>39</v>
@@ -2122,19 +2125,19 @@
         <v>70</v>
       </c>
       <c r="AG2" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AH2" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AI2" s="5" t="s">
         <v>72</v>
       </c>
       <c r="AJ2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK2" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK2" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL2" s="5" t="s">
         <v>39</v>
@@ -2167,13 +2170,13 @@
         <v>0.21</v>
       </c>
       <c r="AV2" s="5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AW2" s="7">
         <v>1.4</v>
       </c>
       <c r="AX2" s="7">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="AY2" s="7">
         <v>0.072</v>
@@ -2182,7 +2185,7 @@
         <v>1</v>
       </c>
       <c r="BA2" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB2" s="5" t="s">
         <v>41</v>
@@ -2200,7 +2203,7 @@
         <v>40</v>
       </c>
       <c r="BG2" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH2" s="8">
         <v>46213</v>
@@ -2212,7 +2215,7 @@
         <v>67</v>
       </c>
       <c r="BK2" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BL2" s="5" t="s">
         <v>39</v>
@@ -2236,7 +2239,7 @@
         <v>71</v>
       </c>
       <c r="BS2" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:71" x14ac:dyDescent="0.25">
@@ -2244,7 +2247,7 @@
         <v>39</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>45</v>
@@ -2298,16 +2301,16 @@
         <v>39</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X3" s="5" t="s">
         <v>39</v>
@@ -2316,7 +2319,7 @@
         <v>39</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA3" s="5" t="s">
         <v>39</v>
@@ -2325,10 +2328,10 @@
         <v>39</v>
       </c>
       <c r="AC3" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AD3" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE3" s="5" t="s">
         <v>39</v>
@@ -2337,19 +2340,19 @@
         <v>70</v>
       </c>
       <c r="AG3" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AH3" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AI3" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AJ3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK3" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK3" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL3" s="5" t="s">
         <v>39</v>
@@ -2382,13 +2385,13 @@
         <v>0.21</v>
       </c>
       <c r="AV3" s="5">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="AW3" s="7">
         <v>1.4</v>
       </c>
       <c r="AX3" s="7">
-        <v>0</v>
+        <v>7.98</v>
       </c>
       <c r="AY3" s="7">
         <v>0.072</v>
@@ -2397,7 +2400,7 @@
         <v>1</v>
       </c>
       <c r="BA3" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB3" s="5" t="s">
         <v>41</v>
@@ -2415,7 +2418,7 @@
         <v>40</v>
       </c>
       <c r="BG3" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH3" s="8">
         <v>46213</v>
@@ -2427,7 +2430,7 @@
         <v>67</v>
       </c>
       <c r="BK3" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BL3" s="5" t="s">
         <v>39</v>
@@ -2451,7 +2454,7 @@
         <v>71</v>
       </c>
       <c r="BS3" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:71" x14ac:dyDescent="0.25">
@@ -2459,7 +2462,7 @@
         <v>39</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>45</v>
@@ -2513,16 +2516,16 @@
         <v>39</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X4" s="5" t="s">
         <v>39</v>
@@ -2531,7 +2534,7 @@
         <v>39</v>
       </c>
       <c r="Z4" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA4" s="5" t="s">
         <v>39</v>
@@ -2540,10 +2543,10 @@
         <v>39</v>
       </c>
       <c r="AC4" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AD4" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE4" s="5" t="s">
         <v>39</v>
@@ -2552,19 +2555,19 @@
         <v>70</v>
       </c>
       <c r="AG4" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AH4" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AI4" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AJ4" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK4" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK4" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL4" s="5" t="s">
         <v>39</v>
@@ -2597,13 +2600,13 @@
         <v>0.21</v>
       </c>
       <c r="AV4" s="5">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AW4" s="7">
         <v>1.4</v>
       </c>
       <c r="AX4" s="7">
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="AY4" s="7">
         <v>0.072</v>
@@ -2612,7 +2615,7 @@
         <v>1</v>
       </c>
       <c r="BA4" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB4" s="5" t="s">
         <v>41</v>
@@ -2630,7 +2633,7 @@
         <v>40</v>
       </c>
       <c r="BG4" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH4" s="8">
         <v>46213</v>
@@ -2642,7 +2645,7 @@
         <v>67</v>
       </c>
       <c r="BK4" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BL4" s="5" t="s">
         <v>39</v>
@@ -2666,7 +2669,7 @@
         <v>71</v>
       </c>
       <c r="BS4" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:71" x14ac:dyDescent="0.25">
@@ -2674,7 +2677,7 @@
         <v>39</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>45</v>
@@ -2728,16 +2731,16 @@
         <v>39</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="X5" s="5" t="s">
         <v>39</v>
@@ -2746,7 +2749,7 @@
         <v>39</v>
       </c>
       <c r="Z5" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA5" s="5" t="s">
         <v>39</v>
@@ -2755,10 +2758,10 @@
         <v>39</v>
       </c>
       <c r="AC5" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AD5" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE5" s="5" t="s">
         <v>39</v>
@@ -2767,19 +2770,19 @@
         <v>70</v>
       </c>
       <c r="AG5" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AH5" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AI5" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AJ5" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK5" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK5" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL5" s="5" t="s">
         <v>39</v>
@@ -2812,13 +2815,13 @@
         <v>0.21</v>
       </c>
       <c r="AV5" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW5" s="7">
         <v>1.4</v>
       </c>
       <c r="AX5" s="7">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="AY5" s="7">
         <v>0.072</v>
@@ -2827,7 +2830,7 @@
         <v>1</v>
       </c>
       <c r="BA5" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB5" s="5" t="s">
         <v>41</v>
@@ -2845,7 +2848,7 @@
         <v>40</v>
       </c>
       <c r="BG5" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH5" s="8">
         <v>46213</v>
@@ -2857,7 +2860,7 @@
         <v>67</v>
       </c>
       <c r="BK5" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BL5" s="5" t="s">
         <v>39</v>
@@ -2881,7 +2884,7 @@
         <v>71</v>
       </c>
       <c r="BS5" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:71" x14ac:dyDescent="0.25">
@@ -2889,13 +2892,13 @@
         <v>39</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E6" s="5" t="b">
         <v>1</v>
@@ -2943,16 +2946,16 @@
         <v>39</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="X6" s="5" t="s">
         <v>39</v>
@@ -2961,19 +2964,19 @@
         <v>39</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AA6" s="5" t="s">
         <v>39</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AC6" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE6" s="5" t="s">
         <v>39</v>
@@ -2982,19 +2985,19 @@
         <v>70</v>
       </c>
       <c r="AG6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AH6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AI6" s="5" t="s">
         <v>72</v>
       </c>
       <c r="AJ6" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK6" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK6" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL6" s="5" t="s">
         <v>39</v>
@@ -3027,13 +3030,13 @@
         <v>0.21</v>
       </c>
       <c r="AV6" s="5">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AW6" s="7">
         <v>1.4</v>
       </c>
       <c r="AX6" s="7">
-        <v>0</v>
+        <v>4.62</v>
       </c>
       <c r="AY6" s="7">
         <v>0.072</v>
@@ -3042,7 +3045,7 @@
         <v>1</v>
       </c>
       <c r="BA6" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB6" s="5" t="s">
         <v>41</v>
@@ -3060,7 +3063,7 @@
         <v>40</v>
       </c>
       <c r="BG6" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH6" s="8">
         <v>46213</v>
@@ -3069,10 +3072,10 @@
         <v>46213</v>
       </c>
       <c r="BJ6" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="BK6" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BL6" s="5" t="s">
         <v>39</v>
@@ -3096,7 +3099,7 @@
         <v>71</v>
       </c>
       <c r="BS6" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:71" x14ac:dyDescent="0.25">
@@ -3104,13 +3107,13 @@
         <v>39</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E7" s="5" t="b">
         <v>1</v>
@@ -3158,16 +3161,16 @@
         <v>39</v>
       </c>
       <c r="T7" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="V7" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="X7" s="5" t="s">
         <v>39</v>
@@ -3176,19 +3179,19 @@
         <v>39</v>
       </c>
       <c r="Z7" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AA7" s="5" t="s">
         <v>39</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AC7" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AD7" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE7" s="5" t="s">
         <v>39</v>
@@ -3197,19 +3200,19 @@
         <v>70</v>
       </c>
       <c r="AG7" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AH7" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AI7" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AJ7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK7" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK7" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL7" s="5" t="s">
         <v>39</v>
@@ -3242,13 +3245,13 @@
         <v>0.21</v>
       </c>
       <c r="AV7" s="5">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="AW7" s="7">
         <v>1.4</v>
       </c>
       <c r="AX7" s="7">
-        <v>0</v>
+        <v>7.56</v>
       </c>
       <c r="AY7" s="7">
         <v>0.072</v>
@@ -3257,7 +3260,7 @@
         <v>1</v>
       </c>
       <c r="BA7" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB7" s="5" t="s">
         <v>41</v>
@@ -3275,7 +3278,7 @@
         <v>40</v>
       </c>
       <c r="BG7" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH7" s="8">
         <v>46213</v>
@@ -3284,10 +3287,10 @@
         <v>46213</v>
       </c>
       <c r="BJ7" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="BK7" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BL7" s="5" t="s">
         <v>39</v>
@@ -3311,7 +3314,7 @@
         <v>71</v>
       </c>
       <c r="BS7" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:71" x14ac:dyDescent="0.25">
@@ -3319,13 +3322,13 @@
         <v>39</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E8" s="5" t="b">
         <v>1</v>
@@ -3373,16 +3376,16 @@
         <v>39</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="V8" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="X8" s="5" t="s">
         <v>39</v>
@@ -3391,19 +3394,19 @@
         <v>39</v>
       </c>
       <c r="Z8" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AA8" s="5" t="s">
         <v>39</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AC8" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AD8" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE8" s="5" t="s">
         <v>39</v>
@@ -3412,19 +3415,19 @@
         <v>70</v>
       </c>
       <c r="AG8" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AH8" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AI8" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AJ8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK8" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK8" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL8" s="5" t="s">
         <v>39</v>
@@ -3457,13 +3460,13 @@
         <v>0.21</v>
       </c>
       <c r="AV8" s="5">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="AW8" s="7">
         <v>1.4</v>
       </c>
       <c r="AX8" s="7">
-        <v>0</v>
+        <v>8.19</v>
       </c>
       <c r="AY8" s="7">
         <v>0.072</v>
@@ -3472,7 +3475,7 @@
         <v>1</v>
       </c>
       <c r="BA8" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB8" s="5" t="s">
         <v>41</v>
@@ -3490,7 +3493,7 @@
         <v>40</v>
       </c>
       <c r="BG8" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH8" s="8">
         <v>46213</v>
@@ -3499,10 +3502,10 @@
         <v>46213</v>
       </c>
       <c r="BJ8" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="BK8" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BL8" s="5" t="s">
         <v>39</v>
@@ -3526,7 +3529,7 @@
         <v>71</v>
       </c>
       <c r="BS8" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:71" x14ac:dyDescent="0.25">
@@ -3534,13 +3537,13 @@
         <v>39</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E9" s="5" t="b">
         <v>1</v>
@@ -3588,16 +3591,16 @@
         <v>39</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="X9" s="5" t="s">
         <v>39</v>
@@ -3606,19 +3609,19 @@
         <v>39</v>
       </c>
       <c r="Z9" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AA9" s="5" t="s">
         <v>39</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AC9" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AD9" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AE9" s="5" t="s">
         <v>39</v>
@@ -3627,19 +3630,19 @@
         <v>70</v>
       </c>
       <c r="AG9" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AH9" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AI9" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AJ9" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK9" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="AK9" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="AL9" s="5" t="s">
         <v>39</v>
@@ -3672,13 +3675,13 @@
         <v>0.21</v>
       </c>
       <c r="AV9" s="5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AW9" s="7">
         <v>1.4</v>
       </c>
       <c r="AX9" s="7">
-        <v>0</v>
+        <v>0.63</v>
       </c>
       <c r="AY9" s="7">
         <v>0.072</v>
@@ -3687,7 +3690,7 @@
         <v>1</v>
       </c>
       <c r="BA9" s="5">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="BB9" s="5" t="s">
         <v>41</v>
@@ -3705,7 +3708,7 @@
         <v>40</v>
       </c>
       <c r="BG9" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BH9" s="8">
         <v>46213</v>
@@ -3714,10 +3717,10 @@
         <v>46213</v>
       </c>
       <c r="BJ9" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="BK9" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BL9" s="5" t="s">
         <v>39</v>
@@ -3741,7 +3744,7 @@
         <v>71</v>
       </c>
       <c r="BS9" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -3763,16 +3766,16 @@
         <v>19</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3794,7 +3797,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -3811,7 +3814,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -3828,7 +3831,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3845,7 +3848,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -3862,7 +3865,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -3879,7 +3882,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -3896,7 +3899,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -3913,7 +3916,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -3930,7 +3933,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -3947,7 +3950,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -3964,7 +3967,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -3981,7 +3984,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -3998,7 +4001,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -4015,7 +4018,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -4032,7 +4035,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -4049,7 +4052,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B18">
         <v>0.7</v>
@@ -4066,12 +4069,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -4082,7 +4085,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -4090,22 +4093,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6285,6 +6288,86 @@
         <v>39</v>
       </c>
       <c r="F110" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>39</v>
+      </c>
+      <c r="B111" t="s">
+        <v>39</v>
+      </c>
+      <c r="C111" t="s">
+        <v>39</v>
+      </c>
+      <c r="D111" t="s">
+        <v>39</v>
+      </c>
+      <c r="E111" t="s">
+        <v>39</v>
+      </c>
+      <c r="F111" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>39</v>
+      </c>
+      <c r="B112" t="s">
+        <v>39</v>
+      </c>
+      <c r="C112" t="s">
+        <v>39</v>
+      </c>
+      <c r="D112" t="s">
+        <v>39</v>
+      </c>
+      <c r="E112" t="s">
+        <v>39</v>
+      </c>
+      <c r="F112" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>39</v>
+      </c>
+      <c r="B113" t="s">
+        <v>39</v>
+      </c>
+      <c r="C113" t="s">
+        <v>39</v>
+      </c>
+      <c r="D113" t="s">
+        <v>39</v>
+      </c>
+      <c r="E113" t="s">
+        <v>39</v>
+      </c>
+      <c r="F113" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>39</v>
+      </c>
+      <c r="B114" t="s">
+        <v>39</v>
+      </c>
+      <c r="C114" t="s">
+        <v>39</v>
+      </c>
+      <c r="D114" t="s">
+        <v>39</v>
+      </c>
+      <c r="E114" t="s">
+        <v>39</v>
+      </c>
+      <c r="F114" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>